<commit_message>
Optimize Selenium test assertions, phone case matching, and click targets
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="339">
   <si>
     <t>Metric</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>22/7/2026</t>
+    <t>20/8/2026</t>
   </si>
   <si>
     <t>Environment</t>
@@ -50,13 +50,13 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>70.00%</t>
+    <t>76.67%</t>
   </si>
   <si>
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>204.26s</t>
+    <t>407.41s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -98,13 +98,13 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-07-22T03:07:58.099Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:44.786Z</t>
-  </si>
-  <si>
-    <t>46.69s</t>
+    <t>2026-08-20T08:55:04.557Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:09.025Z</t>
+  </si>
+  <si>
+    <t>4.47s</t>
   </si>
   <si>
     <t>TC002</t>
@@ -113,13 +113,13 @@
     <t>[TC002] Login with invalid credentials</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:45.020Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:47.011Z</t>
-  </si>
-  <si>
-    <t>1.99s</t>
+    <t>2026-08-20T08:55:19.017Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:23.537Z</t>
+  </si>
+  <si>
+    <t>4.52s</t>
   </si>
   <si>
     <t>TC003</t>
@@ -128,13 +128,13 @@
     <t>[TC003] Login with empty email</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:47.418Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:49.317Z</t>
-  </si>
-  <si>
-    <t>1.90s</t>
+    <t>2026-08-20T08:55:39.777Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:43.854Z</t>
+  </si>
+  <si>
+    <t>4.08s</t>
   </si>
   <si>
     <t>TC004</t>
@@ -143,13 +143,13 @@
     <t>[TC004] Login with empty password</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:49.527Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:51.258Z</t>
-  </si>
-  <si>
-    <t>1.73s</t>
+    <t>2026-08-20T08:55:49.427Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:53.960Z</t>
+  </si>
+  <si>
+    <t>4.53s</t>
   </si>
   <si>
     <t>TC005</t>
@@ -158,13 +158,13 @@
     <t>[TC005] Forgot password flow</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:51.617Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:53.782Z</t>
-  </si>
-  <si>
-    <t>2.17s</t>
+    <t>2026-08-20T08:56:02.490Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:08.706Z</t>
+  </si>
+  <si>
+    <t>6.22s</t>
   </si>
   <si>
     <t>TC006</t>
@@ -176,13 +176,16 @@
     <t>[TC006] Register with valid details</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:54.346Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:56.900Z</t>
-  </si>
-  <si>
-    <t>2.55s</t>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:18.518Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:28.052Z</t>
+  </si>
+  <si>
+    <t>8.55s</t>
   </si>
   <si>
     <t>TC007</t>
@@ -191,13 +194,13 @@
     <t>[TC007] Register with existing email</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:56.964Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:58.825Z</t>
-  </si>
-  <si>
-    <t>1.86s</t>
+    <t>2026-08-20T08:56:32.242Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:35.695Z</t>
+  </si>
+  <si>
+    <t>3.45s</t>
   </si>
   <si>
     <t>TC008</t>
@@ -206,13 +209,13 @@
     <t>[TC008] Register with invalid email</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:59.092Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:02.323Z</t>
-  </si>
-  <si>
-    <t>3.23s</t>
+    <t>2026-08-20T08:56:42.352Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:47.987Z</t>
+  </si>
+  <si>
+    <t>5.63s</t>
   </si>
   <si>
     <t>TC009</t>
@@ -221,13 +224,13 @@
     <t>[TC009] Register with weak password</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:03.547Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:06.200Z</t>
-  </si>
-  <si>
-    <t>2.65s</t>
+    <t>2026-08-20T08:56:56.794Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:57:08.848Z</t>
+  </si>
+  <si>
+    <t>12.05s</t>
   </si>
   <si>
     <t>TC010</t>
@@ -236,13 +239,13 @@
     <t>[TC010] Register with missing mandatory fields</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:06.346Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:08.709Z</t>
-  </si>
-  <si>
-    <t>2.36s</t>
+    <t>2026-08-20T08:57:14.904Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:57:18.744Z</t>
+  </si>
+  <si>
+    <t>3.84s</t>
   </si>
   <si>
     <t>TC011</t>
@@ -254,16 +257,13 @@
     <t>[TC011] Upload suspicious SMS content</t>
   </si>
   <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:09.132Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:18.008Z</t>
-  </si>
-  <si>
-    <t>8.23s</t>
+    <t>2026-08-20T08:57:32.732Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:57:38.492Z</t>
+  </si>
+  <si>
+    <t>5.02s</t>
   </si>
   <si>
     <t>TC012</t>
@@ -272,13 +272,13 @@
     <t>[TC012] Upload phishing message</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:20.637Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:29.246Z</t>
-  </si>
-  <si>
-    <t>7.92s</t>
+    <t>2026-08-20T08:57:59.429Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:07.393Z</t>
+  </si>
+  <si>
+    <t>7.00s</t>
   </si>
   <si>
     <t>TC013</t>
@@ -287,13 +287,13 @@
     <t>[TC013] Upload safe banking message</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:29.975Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:38.657Z</t>
-  </si>
-  <si>
-    <t>8.39s</t>
+    <t>2026-08-20T08:58:14.750Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:22.863Z</t>
+  </si>
+  <si>
+    <t>7.15s</t>
   </si>
   <si>
     <t>TC014</t>
@@ -302,13 +302,13 @@
     <t>[TC014] Analyze suspicious URL</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:38.725Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:52.228Z</t>
-  </si>
-  <si>
-    <t>12.89s</t>
+    <t>2026-08-20T08:58:30.853Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:39.128Z</t>
+  </si>
+  <si>
+    <t>8.27s</t>
   </si>
   <si>
     <t>TC015</t>
@@ -317,13 +317,13 @@
     <t>[TC015] Analyze known phishing URL</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:52.433Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:05.725Z</t>
-  </si>
-  <si>
-    <t>12.59s</t>
+    <t>2026-08-20T08:58:42.806Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:54.813Z</t>
+  </si>
+  <si>
+    <t>12.01s</t>
   </si>
   <si>
     <t>TC016</t>
@@ -335,13 +335,13 @@
     <t>[TC016] Analyze legitimate phone number</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:05.843Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:14.552Z</t>
-  </si>
-  <si>
-    <t>7.83s</t>
+    <t>2026-08-20T08:59:05.852Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:14.284Z</t>
+  </si>
+  <si>
+    <t>8.43s</t>
   </si>
   <si>
     <t>TC017</t>
@@ -350,13 +350,13 @@
     <t>[TC017] Analyze spam caller number</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:15.257Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:23.731Z</t>
-  </si>
-  <si>
-    <t>7.70s</t>
+    <t>2026-08-20T08:59:24.302Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:29.076Z</t>
+  </si>
+  <si>
+    <t>4.77s</t>
   </si>
   <si>
     <t>TC018</t>
@@ -365,13 +365,13 @@
     <t>[TC018] Analyze unknown caller</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:24.143Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:33.481Z</t>
-  </si>
-  <si>
-    <t>8.62s</t>
+    <t>2026-08-20T08:59:37.202Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:43.560Z</t>
+  </si>
+  <si>
+    <t>5.84s</t>
   </si>
   <si>
     <t>TC019</t>
@@ -380,13 +380,13 @@
     <t>[TC019] Block suspicious caller</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:33.973Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:37.695Z</t>
-  </si>
-  <si>
-    <t>2.89s</t>
+    <t>2026-08-20T08:59:47.981Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:55.062Z</t>
+  </si>
+  <si>
+    <t>7.08s</t>
   </si>
   <si>
     <t>TC020</t>
@@ -395,13 +395,13 @@
     <t>[TC020] View call analysis history</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:37.755Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:40.794Z</t>
-  </si>
-  <si>
-    <t>3.04s</t>
+    <t>2026-08-20T09:00:03.872Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:09.073Z</t>
+  </si>
+  <si>
+    <t>5.20s</t>
   </si>
   <si>
     <t>TC021</t>
@@ -413,10 +413,13 @@
     <t>[TC021] Open fraud awareness page</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:41.310Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:43.304Z</t>
+    <t>2026-08-20T09:00:15.661Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:21.459Z</t>
+  </si>
+  <si>
+    <t>5.80s</t>
   </si>
   <si>
     <t>TC022</t>
@@ -425,13 +428,13 @@
     <t>[TC022] Load educational content</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:43.359Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:46.082Z</t>
-  </si>
-  <si>
-    <t>2.72s</t>
+    <t>2026-08-20T09:00:35.002Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:40.734Z</t>
+  </si>
+  <si>
+    <t>5.73s</t>
   </si>
   <si>
     <t>TC023</t>
@@ -440,13 +443,13 @@
     <t>[TC023] Play awareness video</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:46.338Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:49.465Z</t>
-  </si>
-  <si>
-    <t>3.13s</t>
+    <t>2026-08-20T09:00:46.475Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:51.568Z</t>
+  </si>
+  <si>
+    <t>5.09s</t>
   </si>
   <si>
     <t>TC024</t>
@@ -455,13 +458,13 @@
     <t>[TC024] Search awareness topics</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:49.564Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:51.944Z</t>
-  </si>
-  <si>
-    <t>2.38s</t>
+    <t>2026-08-20T09:01:00.217Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:04.270Z</t>
+  </si>
+  <si>
+    <t>3.50s</t>
   </si>
   <si>
     <t>TC025</t>
@@ -470,13 +473,13 @@
     <t>[TC025] Bookmark awareness article</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:53.086Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:56.534Z</t>
-  </si>
-  <si>
-    <t>3.45s</t>
+    <t>2026-08-20T09:01:04.513Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:09.018Z</t>
+  </si>
+  <si>
+    <t>4.50s</t>
   </si>
   <si>
     <t>TC026</t>
@@ -488,13 +491,13 @@
     <t>[TC026] Dashboard loads successfully</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:56.686Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:59.010Z</t>
-  </si>
-  <si>
-    <t>2.32s</t>
+    <t>2026-08-20T09:01:13.395Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:17.801Z</t>
+  </si>
+  <si>
+    <t>4.41s</t>
   </si>
   <si>
     <t>TC027</t>
@@ -503,13 +506,13 @@
     <t>[TC027] Threat statistics displayed</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:59.197Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:01.874Z</t>
-  </si>
-  <si>
-    <t>2.68s</t>
+    <t>2026-08-20T09:01:18.856Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:23.136Z</t>
+  </si>
+  <si>
+    <t>4.28s</t>
   </si>
   <si>
     <t>TC028</t>
@@ -518,10 +521,13 @@
     <t>[TC028] Filter analytics</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:02.012Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:04.369Z</t>
+    <t>2026-08-20T09:01:25.063Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:29.250Z</t>
+  </si>
+  <si>
+    <t>4.19s</t>
   </si>
   <si>
     <t>TC029</t>
@@ -530,13 +536,13 @@
     <t>[TC029] Monthly fraud report loads</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:04.463Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:13.446Z</t>
-  </si>
-  <si>
-    <t>8.98s</t>
+    <t>2026-08-20T09:01:31.488Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:37.380Z</t>
+  </si>
+  <si>
+    <t>5.46s</t>
   </si>
   <si>
     <t>TC030</t>
@@ -545,13 +551,13 @@
     <t>[TC030] Export analytics report</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:18.822Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:22.132Z</t>
-  </si>
-  <si>
-    <t>3.31s</t>
+    <t>2026-08-20T09:01:42.797Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:46.971Z</t>
+  </si>
+  <si>
+    <t>4.17s</t>
   </si>
   <si>
     <t>Failure Reason</t>
@@ -563,51 +569,53 @@
     <t>URL</t>
   </si>
   <si>
+    <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787216187076.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/dashboard</t>
+  </si>
+  <si>
     <t>expected false to be true</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1784689757360.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787216257757.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1784689768554.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1784689778364.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
-Wait timed out after 10228ms</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC014__Analyze_suspicious_URL_1784689791614.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
-Wait timed out after 10060ms</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC015__Analyze_known_phishing_URL_1784689805020.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC016__Analyze_legitimate_phone_number_1784689813675.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787216286428.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787216301905.png</t>
+  </si>
+  <si>
+    <t>expected 'Phone number +91 70135 66677 marked a…' to include 'Marked as'</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC018__Analyze_unknown_caller_1787216383044.png</t>
   </si>
   <si>
     <t>http://localhost:5173/call-analyzer</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC017__Analyze_spam_caller_number_1784689822962.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC018__Analyze_unknown_caller_1784689832765.png</t>
-  </si>
-  <si>
-    <t>expected '+91 98765 43210 SPAM LOAN OFFERS 2026…' to include '+91 99999 00000'</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC019__Block_suspicious_caller_1784689836863.png</t>
+    <t>expected 'Interactive Video Lesson: Spotting UP…' to include 'OTP'</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_5__Banking_Awareness__TC024__Search_awareness_topics_1787216463717.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/awareness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element click intercepted: Element &lt;button id="load-report-btn" class="btn btn-primary" style="padding: 8px 16px;"&gt;...&lt;/button&gt; is not clickable at point (1665, 966). Other element would receive the click: &lt;div class="bottom-nav-bar" data-testid="bottom_nav" style="position: fixed; bottom: 0px; left: 0px; right: 0px; height: 65px; background: rgba(10, 15, 30, 0.95); border-top: 1px solid rgba(255, 255, 255, 0.1); display: flex; align-items: center; z-index: 999; backdrop-filter: blur(16px);"&gt;...&lt;/div&gt;
+  (Session info: chrome=151.0.7922.138)</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_6__Dashboard___Analytics__TC029__Monthly_fraud_report_loads_1787216496954.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -625,7 +633,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:43.994Z</t>
+    <t>2026-08-20T08:55:06.601Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -637,357 +645,381 @@
     <t/>
   </si>
   <si>
-    <t>2026-07-22T03:08:44.719Z</t>
+    <t>2026-08-20T08:55:08.891Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:44.784Z</t>
+    <t>2026-08-20T08:55:09.023Z</t>
   </si>
   <si>
     <t>Successfully verified redirect to Dashboard</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:46.063Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:46.925Z</t>
+    <t>2026-08-20T08:55:21.975Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:22.843Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:47.010Z</t>
+    <t>2026-08-20T08:55:23.536Z</t>
   </si>
   <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:48.689Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:49.165Z</t>
+    <t>2026-08-20T08:55:42.873Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:43.689Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:49.316Z</t>
-  </si>
-  <si>
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:50.704Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:51.183Z</t>
+    <t>2026-08-20T08:55:52.954Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:55:53.847Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
+    <t>2026-08-20T08:55:53.959Z</t>
+  </si>
+  <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:52.698Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:53.707Z</t>
+    <t>2026-08-20T08:56:05.698Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:07.688Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:53.781Z</t>
+    <t>2026-08-20T08:56:08.705Z</t>
   </si>
   <si>
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:55.915Z</t>
+    <t>2026-08-20T08:56:23.653Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:56.894Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_87862@safebank.ai</t>
-  </si>
-  <si>
-    <t>Redirected to Dashboard after secure signup</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:57.950Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:08:58.724Z</t>
+    <t>2026-08-20T08:56:27.015Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_15854@safebank.ai</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:34.198Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:35.371Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
-    <t>2026-07-22T03:08:58.824Z</t>
+    <t>2026-08-20T08:56:35.694Z</t>
   </si>
   <si>
     <t>Verified duplicate email registration error</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:01.086Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:02.236Z</t>
+    <t>2026-08-20T08:56:46.450Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:56:47.835Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:02.322Z</t>
+    <t>2026-08-20T08:56:47.986Z</t>
   </si>
   <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:04.818Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:06.082Z</t>
+    <t>2026-08-20T08:57:07.102Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:57:08.705Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:06.199Z</t>
+    <t>2026-08-20T08:57:08.847Z</t>
   </si>
   <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:07.730Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:08.545Z</t>
+    <t>2026-08-20T08:57:17.840Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:57:18.560Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:08.708Z</t>
+    <t>2026-08-20T08:57:18.743Z</t>
   </si>
   <si>
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:11.413Z</t>
+    <t>2026-08-20T08:57:36.737Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:12.199Z</t>
+    <t>2026-08-20T08:57:37.702Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:22.755Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:23.384Z</t>
+    <t>2026-08-20T08:58:04.957Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:06.363Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:32.460Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:33.200Z</t>
+    <t>2026-08-20T08:58:20.380Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:21.818Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-07-22T03:09:41.034Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:09:54.610Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:08.040Z</t>
+    <t>2026-08-20T08:58:36.811Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:38.367Z</t>
+  </si>
+  <si>
+    <t>Submitted suspicious URL for analysis</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:39.127Z</t>
+  </si>
+  <si>
+    <t>Verified URL threat analysis completes successfully</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:51.735Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:54.010Z</t>
+  </si>
+  <si>
+    <t>Submitted known phishing link URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:58:54.812Z</t>
+  </si>
+  <si>
+    <t>Verified malicious threat flag alert triggers</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:10.971Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:08.568Z</t>
+    <t>2026-08-20T08:59:13.354Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:17.371Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:17.932Z</t>
+    <t>2026-08-20T08:59:14.283Z</t>
+  </si>
+  <si>
+    <t>Verified legitimate number marked Safe</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:27.670Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:28.287Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:27.275Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:27.735Z</t>
+    <t>2026-08-20T08:59:29.075Z</t>
+  </si>
+  <si>
+    <t>Verified spam preset marked Suspicious</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:41.324Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:42.248Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:36.295Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:36.803Z</t>
+    <t>2026-08-20T08:59:53.424Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T08:59:54.953Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:40.002Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:40.545Z</t>
+    <t>Verified number successfully appended to Blocked List table</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:07.402Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:08.205Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
+    <t>2026-08-20T09:00:09.072Z</t>
+  </si>
+  <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:43.296Z</t>
+    <t>2026-08-20T09:00:21.413Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:43.303Z</t>
+    <t>2026-08-20T09:00:21.458Z</t>
   </si>
   <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:45.487Z</t>
+    <t>2026-08-20T09:00:40.124Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:48.647Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:49.374Z</t>
+    <t>2026-08-20T09:00:50.727Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:00:51.446Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:49.464Z</t>
+    <t>2026-08-20T09:00:51.567Z</t>
   </si>
   <si>
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:51.535Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:51.916Z</t>
+    <t>2026-08-20T09:01:02.965Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:03.673Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
   </si>
   <si>
-    <t>Verified articles list filtered based on search query</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:55.172Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:10:56.392Z</t>
+    <t>2026-08-20T09:01:07.664Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:08.895Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:56.533Z</t>
+    <t>2026-08-20T09:01:09.017Z</t>
   </si>
   <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:58.967Z</t>
+    <t>2026-08-20T09:01:17.760Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
-    <t>2026-07-22T03:10:59.009Z</t>
+    <t>2026-08-20T09:01:17.800Z</t>
   </si>
   <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:01.654Z</t>
+    <t>2026-08-20T09:01:22.890Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:23.135Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:04.064Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:04.294Z</t>
+    <t>2026-08-20T09:01:28.914Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:29.166Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:04.368Z</t>
-  </si>
-  <si>
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-07-22T03:11:06.597Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:07.240Z</t>
-  </si>
-  <si>
-    <t>Opened monthly report modal</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:07.891Z</t>
-  </si>
-  <si>
-    <t>Closed monthly report modal</t>
-  </si>
-  <si>
-    <t>Verified monthly intelligence report toggle details</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:21.102Z</t>
-  </si>
-  <si>
-    <t>2026-07-22T03:11:21.906Z</t>
+    <t>2026-08-20T09:01:35.250Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:46.153Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:01:46.817Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
   </si>
   <si>
+    <t>2026-08-20T09:01:46.970Z</t>
+  </si>
+  <si>
     <t>Verified analytics export triggers download confirmation banner</t>
   </si>
   <si>
@@ -1000,7 +1032,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>180.55s</t>
+    <t>175.27s</t>
   </si>
 </sst>
 </file>
@@ -1505,7 +1537,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1513,7 +1545,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1728,28 +1760,28 @@
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>26</v>
+      <c r="E7" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>25</v>
@@ -1758,24 +1790,24 @@
         <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>25</v>
@@ -1784,24 +1816,24 @@
         <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>25</v>
@@ -1810,24 +1842,24 @@
         <v>26</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>25</v>
@@ -1836,30 +1868,30 @@
         <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>80</v>
@@ -1876,7 +1908,7 @@
         <v>83</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>84</v>
@@ -1885,7 +1917,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>85</v>
@@ -1902,7 +1934,7 @@
         <v>88</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>89</v>
@@ -1911,7 +1943,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>90</v>
@@ -1928,7 +1960,7 @@
         <v>93</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>94</v>
@@ -1936,8 +1968,8 @@
       <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>79</v>
+      <c r="E15" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>95</v>
@@ -1954,7 +1986,7 @@
         <v>98</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>99</v>
@@ -1962,8 +1994,8 @@
       <c r="D16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>79</v>
+      <c r="E16" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>100</v>
@@ -1988,8 +2020,8 @@
       <c r="D17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>79</v>
+      <c r="E17" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>106</v>
@@ -2014,8 +2046,8 @@
       <c r="D18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>79</v>
+      <c r="E18" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>111</v>
@@ -2041,7 +2073,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>116</v>
@@ -2066,8 +2098,8 @@
       <c r="D20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="4" t="s">
-        <v>79</v>
+      <c r="E20" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>121</v>
@@ -2128,18 +2160,18 @@
         <v>133</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>34</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>130</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>25</v>
@@ -2148,24 +2180,24 @@
         <v>26</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>130</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>25</v>
@@ -2174,50 +2206,50 @@
         <v>26</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>130</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>26</v>
+      <c r="E25" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>130</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>25</v>
@@ -2226,24 +2258,24 @@
         <v>26</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>25</v>
@@ -2252,24 +2284,24 @@
         <v>26</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>25</v>
@@ -2278,24 +2310,24 @@
         <v>26</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>25</v>
@@ -2304,50 +2336,50 @@
         <v>26</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>75</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>26</v>
+      <c r="E30" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>25</v>
@@ -2356,13 +2388,13 @@
         <v>26</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2373,7 +2405,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2387,169 +2419,135 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>187</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>109</v>
+        <v>171</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2560,7 +2558,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2572,1311 +2570,1345 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>218</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>225</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>236</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>233</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>230</v>
+        <v>253</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>257</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>127</v>
+        <v>288</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>287</v>
+        <v>122</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>137</v>
+        <v>294</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>163</v>
+        <v>314</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D70" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>172</v>
+        <v>326</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>320</v>
+        <v>169</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>304</v>
+        <v>328</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>204</v>
+        <v>26</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B77" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="C77" s="2" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3899,7 +3931,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3908,10 +3940,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>325</v>
+        <v>336</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>326</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3922,16 +3954,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upgrade AI Security Assistant with TTS voice readout, auto-speech responses, and quick suggestion chips
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="331">
   <si>
     <t>Metric</t>
   </si>
@@ -50,13 +50,13 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>76.67%</t>
+    <t>66.67%</t>
   </si>
   <si>
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>407.41s</t>
+    <t>209.83s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -95,31 +95,34 @@
     <t>chrome</t>
   </si>
   <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:03.361Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:08.634Z</t>
+  </si>
+  <si>
+    <t>4.24s</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>[TC002] Login with invalid credentials</t>
+  </si>
+  <si>
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:04.557Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:09.025Z</t>
-  </si>
-  <si>
-    <t>4.47s</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>[TC002] Login with invalid credentials</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:19.017Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:23.537Z</t>
-  </si>
-  <si>
-    <t>4.52s</t>
+    <t>2026-08-20T09:07:08.881Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:11.624Z</t>
+  </si>
+  <si>
+    <t>2.74s</t>
   </si>
   <si>
     <t>TC003</t>
@@ -128,328 +131,325 @@
     <t>[TC003] Login with empty email</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:39.777Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:43.854Z</t>
+    <t>2026-08-20T09:07:11.692Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:14.902Z</t>
+  </si>
+  <si>
+    <t>3.21s</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>[TC004] Login with empty password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:15.164Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:17.328Z</t>
+  </si>
+  <si>
+    <t>2.16s</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>[TC005] Forgot password flow</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:17.382Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:19.999Z</t>
+  </si>
+  <si>
+    <t>2.62s</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Module 2: User Registration</t>
+  </si>
+  <si>
+    <t>[TC006] Register with valid details</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:20.183Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:22.863Z</t>
+  </si>
+  <si>
+    <t>2.28s</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>[TC007] Register with existing email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:23.407Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:26.042Z</t>
+  </si>
+  <si>
+    <t>2.63s</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>[TC008] Register with invalid email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:26.444Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:30.752Z</t>
+  </si>
+  <si>
+    <t>4.31s</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>[TC009] Register with weak password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:30.968Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:34.316Z</t>
+  </si>
+  <si>
+    <t>3.35s</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>[TC010] Register with missing mandatory fields</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:34.846Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:38.622Z</t>
+  </si>
+  <si>
+    <t>3.78s</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Module 3: Fraud Alert Detection</t>
+  </si>
+  <si>
+    <t>[TC011] Upload suspicious SMS content</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:38.924Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:48.276Z</t>
+  </si>
+  <si>
+    <t>8.68s</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>[TC012] Upload phishing message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:48.447Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:59.995Z</t>
+  </si>
+  <si>
+    <t>11.08s</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>[TC013] Upload safe banking message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:00.324Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:09.274Z</t>
+  </si>
+  <si>
+    <t>8.13s</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>[TC014] Analyze suspicious URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:09.388Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:29.054Z</t>
+  </si>
+  <si>
+    <t>18.11s</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>[TC015] Analyze known phishing URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:29.195Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:47.394Z</t>
+  </si>
+  <si>
+    <t>17.15s</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Module 4: Safe Call Analysis</t>
+  </si>
+  <si>
+    <t>[TC016] Analyze legitimate phone number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:47.525Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:59.702Z</t>
+  </si>
+  <si>
+    <t>10.27s</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>[TC017] Analyze spam caller number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:59.856Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:12.478Z</t>
+  </si>
+  <si>
+    <t>11.91s</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>[TC018] Analyze unknown caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:12.646Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:17.799Z</t>
+  </si>
+  <si>
+    <t>5.15s</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>[TC019] Block suspicious caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:17.933Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:22.386Z</t>
+  </si>
+  <si>
+    <t>4.45s</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>[TC020] View call analysis history</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:22.521Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:27.862Z</t>
+  </si>
+  <si>
+    <t>5.34s</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Module 5: Banking Awareness</t>
+  </si>
+  <si>
+    <t>[TC021] Open fraud awareness page</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:28.076Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:34.242Z</t>
+  </si>
+  <si>
+    <t>6.17s</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>[TC022] Load educational content</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:34.476Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:38.556Z</t>
   </si>
   <si>
     <t>4.08s</t>
   </si>
   <si>
-    <t>TC004</t>
-  </si>
-  <si>
-    <t>[TC004] Login with empty password</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:49.427Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:53.960Z</t>
-  </si>
-  <si>
-    <t>4.53s</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>[TC005] Forgot password flow</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:02.490Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:08.706Z</t>
-  </si>
-  <si>
-    <t>6.22s</t>
-  </si>
-  <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>Module 2: User Registration</t>
-  </si>
-  <si>
-    <t>[TC006] Register with valid details</t>
-  </si>
-  <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:18.518Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:28.052Z</t>
-  </si>
-  <si>
-    <t>8.55s</t>
-  </si>
-  <si>
-    <t>TC007</t>
-  </si>
-  <si>
-    <t>[TC007] Register with existing email</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:32.242Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:35.695Z</t>
-  </si>
-  <si>
-    <t>3.45s</t>
-  </si>
-  <si>
-    <t>TC008</t>
-  </si>
-  <si>
-    <t>[TC008] Register with invalid email</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:42.352Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:47.987Z</t>
-  </si>
-  <si>
-    <t>5.63s</t>
-  </si>
-  <si>
-    <t>TC009</t>
-  </si>
-  <si>
-    <t>[TC009] Register with weak password</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:56.794Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:08.848Z</t>
-  </si>
-  <si>
-    <t>12.05s</t>
-  </si>
-  <si>
-    <t>TC010</t>
-  </si>
-  <si>
-    <t>[TC010] Register with missing mandatory fields</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:14.904Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:18.744Z</t>
-  </si>
-  <si>
-    <t>3.84s</t>
-  </si>
-  <si>
-    <t>TC011</t>
-  </si>
-  <si>
-    <t>Module 3: Fraud Alert Detection</t>
-  </si>
-  <si>
-    <t>[TC011] Upload suspicious SMS content</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:32.732Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:38.492Z</t>
-  </si>
-  <si>
-    <t>5.02s</t>
-  </si>
-  <si>
-    <t>TC012</t>
-  </si>
-  <si>
-    <t>[TC012] Upload phishing message</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:59.429Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:07.393Z</t>
-  </si>
-  <si>
-    <t>7.00s</t>
-  </si>
-  <si>
-    <t>TC013</t>
-  </si>
-  <si>
-    <t>[TC013] Upload safe banking message</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:14.750Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:22.863Z</t>
-  </si>
-  <si>
-    <t>7.15s</t>
-  </si>
-  <si>
-    <t>TC014</t>
-  </si>
-  <si>
-    <t>[TC014] Analyze suspicious URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:30.853Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:39.128Z</t>
-  </si>
-  <si>
-    <t>8.27s</t>
-  </si>
-  <si>
-    <t>TC015</t>
-  </si>
-  <si>
-    <t>[TC015] Analyze known phishing URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:42.806Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:54.813Z</t>
-  </si>
-  <si>
-    <t>12.01s</t>
-  </si>
-  <si>
-    <t>TC016</t>
-  </si>
-  <si>
-    <t>Module 4: Safe Call Analysis</t>
-  </si>
-  <si>
-    <t>[TC016] Analyze legitimate phone number</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:05.852Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:14.284Z</t>
-  </si>
-  <si>
-    <t>8.43s</t>
-  </si>
-  <si>
-    <t>TC017</t>
-  </si>
-  <si>
-    <t>[TC017] Analyze spam caller number</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:24.302Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:29.076Z</t>
-  </si>
-  <si>
-    <t>4.77s</t>
-  </si>
-  <si>
-    <t>TC018</t>
-  </si>
-  <si>
-    <t>[TC018] Analyze unknown caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:37.202Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:43.560Z</t>
-  </si>
-  <si>
-    <t>5.84s</t>
-  </si>
-  <si>
-    <t>TC019</t>
-  </si>
-  <si>
-    <t>[TC019] Block suspicious caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:47.981Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:55.062Z</t>
-  </si>
-  <si>
-    <t>7.08s</t>
-  </si>
-  <si>
-    <t>TC020</t>
-  </si>
-  <si>
-    <t>[TC020] View call analysis history</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:03.872Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:09.073Z</t>
-  </si>
-  <si>
-    <t>5.20s</t>
-  </si>
-  <si>
-    <t>TC021</t>
-  </si>
-  <si>
-    <t>Module 5: Banking Awareness</t>
-  </si>
-  <si>
-    <t>[TC021] Open fraud awareness page</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:15.661Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:21.459Z</t>
-  </si>
-  <si>
-    <t>5.80s</t>
-  </si>
-  <si>
-    <t>TC022</t>
-  </si>
-  <si>
-    <t>[TC022] Load educational content</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:35.002Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:40.734Z</t>
-  </si>
-  <si>
-    <t>5.73s</t>
-  </si>
-  <si>
     <t>TC023</t>
   </si>
   <si>
     <t>[TC023] Play awareness video</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:46.475Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:51.568Z</t>
-  </si>
-  <si>
-    <t>5.09s</t>
+    <t>2026-08-20T09:09:38.780Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:43.703Z</t>
+  </si>
+  <si>
+    <t>4.92s</t>
   </si>
   <si>
     <t>TC024</t>
@@ -458,13 +458,13 @@
     <t>[TC024] Search awareness topics</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:00.217Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:04.270Z</t>
-  </si>
-  <si>
-    <t>3.50s</t>
+    <t>2026-08-20T09:09:43.829Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:48.856Z</t>
+  </si>
+  <si>
+    <t>5.03s</t>
   </si>
   <si>
     <t>TC025</t>
@@ -473,13 +473,13 @@
     <t>[TC025] Bookmark awareness article</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:04.513Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:09.018Z</t>
-  </si>
-  <si>
-    <t>4.50s</t>
+    <t>2026-08-20T09:09:48.966Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:55.060Z</t>
+  </si>
+  <si>
+    <t>6.09s</t>
   </si>
   <si>
     <t>TC026</t>
@@ -491,13 +491,13 @@
     <t>[TC026] Dashboard loads successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:13.395Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:17.801Z</t>
-  </si>
-  <si>
-    <t>4.41s</t>
+    <t>2026-08-20T09:09:55.153Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:02.668Z</t>
+  </si>
+  <si>
+    <t>7.51s</t>
   </si>
   <si>
     <t>TC027</t>
@@ -506,13 +506,13 @@
     <t>[TC027] Threat statistics displayed</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:18.856Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:23.136Z</t>
-  </si>
-  <si>
-    <t>4.28s</t>
+    <t>2026-08-20T09:10:02.830Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:13.073Z</t>
+  </si>
+  <si>
+    <t>10.24s</t>
   </si>
   <si>
     <t>TC028</t>
@@ -521,13 +521,13 @@
     <t>[TC028] Filter analytics</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:25.063Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:29.250Z</t>
-  </si>
-  <si>
-    <t>4.19s</t>
+    <t>2026-08-20T09:10:13.800Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:19.148Z</t>
+  </si>
+  <si>
+    <t>5.35s</t>
   </si>
   <si>
     <t>TC029</t>
@@ -536,13 +536,13 @@
     <t>[TC029] Monthly fraud report loads</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:31.488Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:37.380Z</t>
-  </si>
-  <si>
-    <t>5.46s</t>
+    <t>2026-08-20T09:10:19.335Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:25.590Z</t>
+  </si>
+  <si>
+    <t>5.69s</t>
   </si>
   <si>
     <t>TC030</t>
@@ -551,13 +551,13 @@
     <t>[TC030] Export analytics report</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:42.797Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:46.971Z</t>
-  </si>
-  <si>
-    <t>4.17s</t>
+    <t>2026-08-20T09:10:25.750Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:32.942Z</t>
+  </si>
+  <si>
+    <t>7.19s</t>
   </si>
   <si>
     <t>Failure Reason</t>
@@ -569,53 +569,61 @@
     <t>URL</t>
   </si>
   <si>
+    <t>expected false to be true</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_1__Authentication__TC001__Login_with_valid_credentials_1787216827605.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/dashboard</t>
+  </si>
+  <si>
     <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787216187076.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/dashboard</t>
-  </si>
-  <si>
-    <t>expected false to be true</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787216257757.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787216842467.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787216867609.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787216286428.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787216301905.png</t>
-  </si>
-  <si>
-    <t>expected 'Phone number +91 70135 66677 marked a…' to include 'Marked as'</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC018__Analyze_unknown_caller_1787216383044.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787216879532.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787216888453.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
+Wait timed out after 10170ms</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC014__Analyze_suspicious_URL_1787216907514.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
+Wait timed out after 10197ms</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC015__Analyze_known_phishing_URL_1787216926351.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC016__Analyze_legitimate_phone_number_1787216937802.png</t>
   </si>
   <si>
     <t>http://localhost:5173/call-analyzer</t>
   </si>
   <si>
-    <t>expected 'Interactive Video Lesson: Spotting UP…' to include 'OTP'</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_5__Banking_Awareness__TC024__Search_awareness_topics_1787216463717.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/awareness</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC017__Analyze_spam_caller_number_1787216951768.png</t>
   </si>
   <si>
     <t xml:space="preserve">element click intercepted: Element &lt;button id="load-report-btn" class="btn btn-primary" style="padding: 8px 16px;"&gt;...&lt;/button&gt; is not clickable at point (1665, 966). Other element would receive the click: &lt;div class="bottom-nav-bar" data-testid="bottom_nav" style="position: fixed; bottom: 0px; left: 0px; right: 0px; height: 65px; background: rgba(10, 15, 30, 0.95); border-top: 1px solid rgba(255, 255, 255, 0.1); display: flex; align-items: center; z-index: 999; backdrop-filter: blur(16px);"&gt;...&lt;/div&gt;
   (Session info: chrome=151.0.7922.138)</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_6__Dashboard___Analytics__TC029__Monthly_fraud_report_loads_1787216496954.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_6__Dashboard___Analytics__TC029__Monthly_fraud_report_loads_1787217025025.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -633,7 +641,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:06.601Z</t>
+    <t>2026-08-20T09:07:06.757Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -645,37 +653,31 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-20T08:55:08.891Z</t>
+    <t>2026-08-20T09:07:07.432Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:09.023Z</t>
-  </si>
-  <si>
-    <t>Successfully verified redirect to Dashboard</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:21.975Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:22.843Z</t>
+    <t>2026-08-20T09:07:10.705Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:11.309Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:23.536Z</t>
+    <t>2026-08-20T09:07:11.623Z</t>
   </si>
   <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:42.873Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:43.689Z</t>
+    <t>2026-08-20T09:07:13.979Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:14.707Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
@@ -684,342 +686,318 @@
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:52.954Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:55:53.847Z</t>
+    <t>2026-08-20T09:07:16.688Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:17.235Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
-    <t>2026-08-20T08:55:53.959Z</t>
+    <t>2026-08-20T09:07:17.327Z</t>
   </si>
   <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:05.698Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:07.688Z</t>
+    <t>2026-08-20T09:07:19.049Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:19.475Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:08.705Z</t>
-  </si>
-  <si>
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:23.653Z</t>
+    <t>2026-08-20T09:07:21.737Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:27.015Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_15854@safebank.ai</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:34.198Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:35.371Z</t>
+    <t>2026-08-20T09:07:22.461Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_2717@safebank.ai</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:24.940Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:25.756Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:35.694Z</t>
+    <t>2026-08-20T09:07:26.041Z</t>
   </si>
   <si>
     <t>Verified duplicate email registration error</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:46.450Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:56:47.835Z</t>
+    <t>2026-08-20T09:07:29.774Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:30.678Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
-    <t>2026-08-20T08:56:47.986Z</t>
-  </si>
-  <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:07.102Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:08.705Z</t>
+    <t>2026-08-20T09:07:32.717Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:34.206Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:08.847Z</t>
+    <t>2026-08-20T09:07:34.315Z</t>
   </si>
   <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:17.840Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:57:18.560Z</t>
+    <t>2026-08-20T09:07:37.669Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:38.434Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:18.743Z</t>
+    <t>2026-08-20T09:07:38.621Z</t>
   </si>
   <si>
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:36.737Z</t>
+    <t>2026-08-20T09:07:41.780Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-08-20T08:57:37.702Z</t>
+    <t>2026-08-20T09:07:42.545Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T08:58:04.957Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:06.363Z</t>
+    <t>2026-08-20T09:07:53.503Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:07:54.320Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T08:58:20.380Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:21.818Z</t>
+    <t>2026-08-20T09:08:02.977Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:03.429Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-08-20T08:58:36.811Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:38.367Z</t>
-  </si>
-  <si>
-    <t>Submitted suspicious URL for analysis</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:39.127Z</t>
-  </si>
-  <si>
-    <t>Verified URL threat analysis completes successfully</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:51.735Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:54.010Z</t>
-  </si>
-  <si>
-    <t>Submitted known phishing link URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:58:54.812Z</t>
-  </si>
-  <si>
-    <t>Verified malicious threat flag alert triggers</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:10.971Z</t>
+    <t>2026-08-20T09:08:16.882Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:35.751Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:08:51.886Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-08-20T08:59:13.354Z</t>
+    <t>2026-08-20T09:08:52.686Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T08:59:14.283Z</t>
-  </si>
-  <si>
-    <t>Verified legitimate number marked Safe</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:27.670Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:28.287Z</t>
+    <t>2026-08-20T09:09:05.846Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:06.628Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T08:59:29.075Z</t>
-  </si>
-  <si>
-    <t>Verified spam preset marked Suspicious</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:41.324Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:42.248Z</t>
+    <t>2026-08-20T09:09:16.128Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:16.962Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T08:59:53.424Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T08:59:54.953Z</t>
+    <t>2026-08-20T09:09:17.798Z</t>
+  </si>
+  <si>
+    <t>Verified call risk assessment generated and shown</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:21.619Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:22.288Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
+    <t>2026-08-20T09:09:22.385Z</t>
+  </si>
+  <si>
     <t>Verified number successfully appended to Blocked List table</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:07.402Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:08.205Z</t>
+    <t>2026-08-20T09:09:25.769Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:26.859Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:09.072Z</t>
+    <t>2026-08-20T09:09:27.861Z</t>
   </si>
   <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:21.413Z</t>
+    <t>2026-08-20T09:09:34.113Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:21.458Z</t>
+    <t>2026-08-20T09:09:34.241Z</t>
   </si>
   <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:40.124Z</t>
+    <t>2026-08-20T09:09:37.969Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:38.555Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:50.727Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:00:51.446Z</t>
+    <t>2026-08-20T09:09:42.816Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:43.560Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
   </si>
   <si>
-    <t>2026-08-20T09:00:51.567Z</t>
+    <t>2026-08-20T09:09:43.700Z</t>
   </si>
   <si>
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:02.965Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:03.673Z</t>
+    <t>2026-08-20T09:09:47.493Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:48.811Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:07.664Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:08.895Z</t>
+    <t>2026-08-20T09:09:48.855Z</t>
+  </si>
+  <si>
+    <t>Verified articles list filtered based on search query</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:53.629Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:09:54.918Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:09.017Z</t>
+    <t>2026-08-20T09:09:55.059Z</t>
   </si>
   <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:17.760Z</t>
+    <t>2026-08-20T09:10:02.606Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:17.800Z</t>
+    <t>2026-08-20T09:10:02.667Z</t>
   </si>
   <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:22.890Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:23.135Z</t>
+    <t>2026-08-20T09:10:12.488Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:13.072Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:28.914Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:29.166Z</t>
+    <t>2026-08-20T09:10:18.685Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:19.053Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
   </si>
   <si>
+    <t>2026-08-20T09:10:19.147Z</t>
+  </si>
+  <si>
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:35.250Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:46.153Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:01:46.817Z</t>
+    <t>2026-08-20T09:10:23.291Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:31.949Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:10:32.748Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
   </si>
   <si>
-    <t>2026-08-20T09:01:46.970Z</t>
-  </si>
-  <si>
     <t>Verified analytics export triggers download confirmation banner</t>
   </si>
   <si>
@@ -1032,7 +1010,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>175.27s</t>
+    <t>193.88s</t>
   </si>
 </sst>
 </file>
@@ -1537,7 +1515,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1545,7 +1523,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1630,7 +1608,7 @@
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1657,111 +1635,111 @@
         <v>25</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>54</v>
@@ -1778,7 +1756,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -1787,7 +1765,7 @@
         <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>59</v>
@@ -1804,7 +1782,7 @@
         <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>63</v>
@@ -1813,7 +1791,7 @@
         <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>64</v>
@@ -1830,7 +1808,7 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>68</v>
@@ -1839,7 +1817,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>69</v>
@@ -1856,7 +1834,7 @@
         <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>73</v>
@@ -1865,7 +1843,7 @@
         <v>25</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>74</v>
@@ -1891,7 +1869,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>80</v>
@@ -1917,7 +1895,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>85</v>
@@ -1943,7 +1921,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>90</v>
@@ -1968,7 +1946,7 @@
       <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -1994,7 +1972,7 @@
       <c r="D16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
@@ -2020,7 +1998,7 @@
       <c r="D17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -2046,7 +2024,7 @@
       <c r="D18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
@@ -2072,8 +2050,8 @@
       <c r="D19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>53</v>
+      <c r="E19" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>116</v>
@@ -2099,7 +2077,7 @@
         <v>25</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>121</v>
@@ -2125,7 +2103,7 @@
         <v>25</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>126</v>
@@ -2151,7 +2129,7 @@
         <v>25</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>132</v>
@@ -2177,7 +2155,7 @@
         <v>25</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>137</v>
@@ -2203,7 +2181,7 @@
         <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>142</v>
@@ -2228,8 +2206,8 @@
       <c r="D25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>53</v>
+      <c r="E25" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>147</v>
@@ -2255,7 +2233,7 @@
         <v>25</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>152</v>
@@ -2281,7 +2259,7 @@
         <v>25</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>158</v>
@@ -2307,7 +2285,7 @@
         <v>25</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>163</v>
@@ -2333,7 +2311,7 @@
         <v>25</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>168</v>
@@ -2359,7 +2337,7 @@
         <v>25</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>173</v>
@@ -2385,7 +2363,7 @@
         <v>25</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>178</v>
@@ -2405,7 +2383,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2433,7 +2411,7 @@
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>184</v>
@@ -2450,7 +2428,7 @@
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>187</v>
@@ -2462,32 +2440,32 @@
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>191</v>
@@ -2496,57 +2474,108 @@
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>193</v>
-      </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="B11" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2558,7 +2587,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2570,308 +2599,308 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>219</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>38</v>
+        <v>222</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>206</v>
+        <v>229</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>228</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2882,47 +2911,47 @@
         <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2933,18 +2962,18 @@
         <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>242</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>63</v>
@@ -2953,10 +2982,10 @@
         <v>243</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2964,33 +2993,33 @@
         <v>244</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3004,10 +3033,10 @@
         <v>248</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3015,33 +3044,33 @@
         <v>249</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3055,10 +3084,10 @@
         <v>253</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3066,16 +3095,16 @@
         <v>254</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>255</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3089,10 +3118,10 @@
         <v>257</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3100,33 +3129,33 @@
         <v>258</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3134,33 +3163,33 @@
         <v>261</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3168,322 +3197,322 @@
         <v>264</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>268</v>
-      </c>
       <c r="D38" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>270</v>
-      </c>
       <c r="D39" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>273</v>
-      </c>
       <c r="D41" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>281</v>
+        <v>267</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>286</v>
+        <v>267</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>292</v>
-      </c>
       <c r="D52" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>122</v>
+        <v>292</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>277</v>
-      </c>
       <c r="D54" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3491,101 +3520,101 @@
         <v>295</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="D56" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>300</v>
-      </c>
       <c r="D57" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>138</v>
+        <v>303</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>304</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3593,16 +3622,16 @@
         <v>305</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3610,16 +3639,16 @@
         <v>306</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>307</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3627,16 +3656,16 @@
         <v>308</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>309</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3644,84 +3673,84 @@
         <v>310</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3729,16 +3758,16 @@
         <v>318</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>319</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3746,16 +3775,16 @@
         <v>320</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>321</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3763,16 +3792,16 @@
         <v>322</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3780,135 +3809,50 @@
         <v>323</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>319</v>
-      </c>
       <c r="D73" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="D74" s="9" t="s">
-        <v>207</v>
+        <v>32</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D76" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="D78" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="D79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -3931,7 +3875,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3940,10 +3884,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3954,16 +3898,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="2">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D2" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Optimize Selenium E2E test handlers and login state checks
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="333">
   <si>
     <t>Metric</t>
   </si>
@@ -50,13 +50,13 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>66.67%</t>
+    <t>86.67%</t>
   </si>
   <si>
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>209.83s</t>
+    <t>181.98s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -95,97 +95,97 @@
     <t>chrome</t>
   </si>
   <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:03.612Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:07.806Z</t>
+  </si>
+  <si>
+    <t>4.19s</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>[TC002] Login with invalid credentials</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:07.886Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:12.204Z</t>
+  </si>
+  <si>
+    <t>4.32s</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>[TC003] Login with empty email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:12.331Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:17.356Z</t>
+  </si>
+  <si>
+    <t>5.02s</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>[TC004] Login with empty password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:17.488Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:20.362Z</t>
+  </si>
+  <si>
+    <t>2.87s</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>[TC005] Forgot password flow</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:20.472Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:25.526Z</t>
+  </si>
+  <si>
+    <t>5.05s</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Module 2: User Registration</t>
+  </si>
+  <si>
+    <t>[TC006] Register with valid details</t>
+  </si>
+  <si>
     <t>FAILED</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:03.361Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:08.634Z</t>
-  </si>
-  <si>
-    <t>4.24s</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>[TC002] Login with invalid credentials</t>
-  </si>
-  <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:08.881Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:11.624Z</t>
-  </si>
-  <si>
-    <t>2.74s</t>
-  </si>
-  <si>
-    <t>TC003</t>
-  </si>
-  <si>
-    <t>[TC003] Login with empty email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:11.692Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:14.902Z</t>
-  </si>
-  <si>
-    <t>3.21s</t>
-  </si>
-  <si>
-    <t>TC004</t>
-  </si>
-  <si>
-    <t>[TC004] Login with empty password</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:15.164Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:17.328Z</t>
-  </si>
-  <si>
-    <t>2.16s</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>[TC005] Forgot password flow</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:17.382Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:19.999Z</t>
-  </si>
-  <si>
-    <t>2.62s</t>
-  </si>
-  <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>Module 2: User Registration</t>
-  </si>
-  <si>
-    <t>[TC006] Register with valid details</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:20.183Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:22.863Z</t>
-  </si>
-  <si>
-    <t>2.28s</t>
+    <t>2026-08-20T09:11:26.566Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:33.759Z</t>
+  </si>
+  <si>
+    <t>5.88s</t>
   </si>
   <si>
     <t>TC007</t>
@@ -194,13 +194,13 @@
     <t>[TC007] Register with existing email</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:23.407Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:26.042Z</t>
-  </si>
-  <si>
-    <t>2.63s</t>
+    <t>2026-08-20T09:11:33.941Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:38.934Z</t>
+  </si>
+  <si>
+    <t>4.99s</t>
   </si>
   <si>
     <t>TC008</t>
@@ -209,13 +209,13 @@
     <t>[TC008] Register with invalid email</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:26.444Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:30.752Z</t>
-  </si>
-  <si>
-    <t>4.31s</t>
+    <t>2026-08-20T09:11:39.200Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:43.714Z</t>
+  </si>
+  <si>
+    <t>4.51s</t>
   </si>
   <si>
     <t>TC009</t>
@@ -224,13 +224,13 @@
     <t>[TC009] Register with weak password</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:30.968Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:34.316Z</t>
-  </si>
-  <si>
-    <t>3.35s</t>
+    <t>2026-08-20T09:11:43.928Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:47.499Z</t>
+  </si>
+  <si>
+    <t>3.57s</t>
   </si>
   <si>
     <t>TC010</t>
@@ -239,13 +239,13 @@
     <t>[TC010] Register with missing mandatory fields</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:34.846Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:38.622Z</t>
-  </si>
-  <si>
-    <t>3.78s</t>
+    <t>2026-08-20T09:11:47.613Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:51.979Z</t>
+  </si>
+  <si>
+    <t>4.37s</t>
   </si>
   <si>
     <t>TC011</t>
@@ -257,13 +257,13 @@
     <t>[TC011] Upload suspicious SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:38.924Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:48.276Z</t>
-  </si>
-  <si>
-    <t>8.68s</t>
+    <t>2026-08-20T09:11:52.167Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:59.358Z</t>
+  </si>
+  <si>
+    <t>6.24s</t>
   </si>
   <si>
     <t>TC012</t>
@@ -272,13 +272,13 @@
     <t>[TC012] Upload phishing message</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:48.447Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:59.995Z</t>
-  </si>
-  <si>
-    <t>11.08s</t>
+    <t>2026-08-20T09:11:59.652Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:08.341Z</t>
+  </si>
+  <si>
+    <t>7.83s</t>
   </si>
   <si>
     <t>TC013</t>
@@ -287,13 +287,13 @@
     <t>[TC013] Upload safe banking message</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:00.324Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:09.274Z</t>
-  </si>
-  <si>
-    <t>8.13s</t>
+    <t>2026-08-20T09:12:08.503Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:15.401Z</t>
+  </si>
+  <si>
+    <t>5.86s</t>
   </si>
   <si>
     <t>TC014</t>
@@ -302,13 +302,13 @@
     <t>[TC014] Analyze suspicious URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:09.388Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:29.054Z</t>
-  </si>
-  <si>
-    <t>18.11s</t>
+    <t>2026-08-20T09:12:15.474Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:23.686Z</t>
+  </si>
+  <si>
+    <t>8.21s</t>
   </si>
   <si>
     <t>TC015</t>
@@ -317,13 +317,13 @@
     <t>[TC015] Analyze known phishing URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:29.195Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:47.394Z</t>
-  </si>
-  <si>
-    <t>17.15s</t>
+    <t>2026-08-20T09:12:23.904Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:29.645Z</t>
+  </si>
+  <si>
+    <t>5.74s</t>
   </si>
   <si>
     <t>TC016</t>
@@ -335,13 +335,13 @@
     <t>[TC016] Analyze legitimate phone number</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:47.525Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:59.702Z</t>
-  </si>
-  <si>
-    <t>10.27s</t>
+    <t>2026-08-20T09:12:29.835Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:34.806Z</t>
+  </si>
+  <si>
+    <t>4.97s</t>
   </si>
   <si>
     <t>TC017</t>
@@ -350,13 +350,13 @@
     <t>[TC017] Analyze spam caller number</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:59.856Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:12.478Z</t>
-  </si>
-  <si>
-    <t>11.91s</t>
+    <t>2026-08-20T09:12:35.060Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:41.600Z</t>
+  </si>
+  <si>
+    <t>6.54s</t>
   </si>
   <si>
     <t>TC018</t>
@@ -365,13 +365,13 @@
     <t>[TC018] Analyze unknown caller</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:12.646Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:17.799Z</t>
-  </si>
-  <si>
-    <t>5.15s</t>
+    <t>2026-08-20T09:12:41.716Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:48.494Z</t>
+  </si>
+  <si>
+    <t>6.78s</t>
   </si>
   <si>
     <t>TC019</t>
@@ -380,13 +380,13 @@
     <t>[TC019] Block suspicious caller</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:17.933Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:22.386Z</t>
-  </si>
-  <si>
-    <t>4.45s</t>
+    <t>2026-08-20T09:12:49.657Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:55.157Z</t>
+  </si>
+  <si>
+    <t>5.50s</t>
   </si>
   <si>
     <t>TC020</t>
@@ -395,13 +395,13 @@
     <t>[TC020] View call analysis history</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:22.521Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:27.862Z</t>
-  </si>
-  <si>
-    <t>5.34s</t>
+    <t>2026-08-20T09:12:55.527Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:00.272Z</t>
+  </si>
+  <si>
+    <t>4.75s</t>
   </si>
   <si>
     <t>TC021</t>
@@ -413,13 +413,13 @@
     <t>[TC021] Open fraud awareness page</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:28.076Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:34.242Z</t>
-  </si>
-  <si>
-    <t>6.17s</t>
+    <t>2026-08-20T09:13:00.344Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:04.394Z</t>
+  </si>
+  <si>
+    <t>4.05s</t>
   </si>
   <si>
     <t>TC022</t>
@@ -428,13 +428,13 @@
     <t>[TC022] Load educational content</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:34.476Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:38.556Z</t>
-  </si>
-  <si>
-    <t>4.08s</t>
+    <t>2026-08-20T09:13:04.647Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:09.449Z</t>
+  </si>
+  <si>
+    <t>4.80s</t>
   </si>
   <si>
     <t>TC023</t>
@@ -443,13 +443,13 @@
     <t>[TC023] Play awareness video</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:38.780Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:43.703Z</t>
-  </si>
-  <si>
-    <t>4.92s</t>
+    <t>2026-08-20T09:13:09.618Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:13.910Z</t>
+  </si>
+  <si>
+    <t>4.29s</t>
   </si>
   <si>
     <t>TC024</t>
@@ -458,13 +458,13 @@
     <t>[TC024] Search awareness topics</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:43.829Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:48.856Z</t>
-  </si>
-  <si>
-    <t>5.03s</t>
+    <t>2026-08-20T09:13:14.053Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:18.145Z</t>
+  </si>
+  <si>
+    <t>4.09s</t>
   </si>
   <si>
     <t>TC025</t>
@@ -473,13 +473,13 @@
     <t>[TC025] Bookmark awareness article</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:48.966Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:55.060Z</t>
-  </si>
-  <si>
-    <t>6.09s</t>
+    <t>2026-08-20T09:13:18.215Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:23.605Z</t>
+  </si>
+  <si>
+    <t>5.39s</t>
   </si>
   <si>
     <t>TC026</t>
@@ -491,13 +491,13 @@
     <t>[TC026] Dashboard loads successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:55.153Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:02.668Z</t>
-  </si>
-  <si>
-    <t>7.51s</t>
+    <t>2026-08-20T09:13:23.994Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:28.512Z</t>
+  </si>
+  <si>
+    <t>4.52s</t>
   </si>
   <si>
     <t>TC027</t>
@@ -506,13 +506,13 @@
     <t>[TC027] Threat statistics displayed</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:02.830Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:13.073Z</t>
-  </si>
-  <si>
-    <t>10.24s</t>
+    <t>2026-08-20T09:13:29.625Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:33.989Z</t>
+  </si>
+  <si>
+    <t>4.36s</t>
   </si>
   <si>
     <t>TC028</t>
@@ -521,13 +521,13 @@
     <t>[TC028] Filter analytics</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:13.800Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:19.148Z</t>
-  </si>
-  <si>
-    <t>5.35s</t>
+    <t>2026-08-20T09:13:34.210Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:38.024Z</t>
+  </si>
+  <si>
+    <t>3.81s</t>
   </si>
   <si>
     <t>TC029</t>
@@ -536,13 +536,13 @@
     <t>[TC029] Monthly fraud report loads</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:19.335Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:25.590Z</t>
-  </si>
-  <si>
-    <t>5.69s</t>
+    <t>2026-08-20T09:13:38.501Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:53.035Z</t>
+  </si>
+  <si>
+    <t>14.53s</t>
   </si>
   <si>
     <t>TC030</t>
@@ -551,13 +551,13 @@
     <t>[TC030] Export analytics report</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:25.750Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:32.942Z</t>
-  </si>
-  <si>
-    <t>7.19s</t>
+    <t>2026-08-20T09:13:53.156Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:14:03.858Z</t>
+  </si>
+  <si>
+    <t>10.70s</t>
   </si>
   <si>
     <t>Failure Reason</t>
@@ -569,61 +569,28 @@
     <t>URL</t>
   </si>
   <si>
+    <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217092451.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/dashboard</t>
+  </si>
+  <si>
     <t>expected false to be true</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_1__Authentication__TC001__Login_with_valid_credentials_1787216827605.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/dashboard</t>
-  </si>
-  <si>
-    <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787216842467.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787216867609.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217118408.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787216879532.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787216888453.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
-Wait timed out after 10170ms</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC014__Analyze_suspicious_URL_1787216907514.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting for element to be located By(css selector, *[id="url-input"])
-Wait timed out after 10197ms</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC015__Analyze_known_phishing_URL_1787216926351.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC016__Analyze_legitimate_phone_number_1787216937802.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/call-analyzer</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_4__Safe_Call_Analysis__TC017__Analyze_spam_caller_number_1787216951768.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">element click intercepted: Element &lt;button id="load-report-btn" class="btn btn-primary" style="padding: 8px 16px;"&gt;...&lt;/button&gt; is not clickable at point (1665, 966). Other element would receive the click: &lt;div class="bottom-nav-bar" data-testid="bottom_nav" style="position: fixed; bottom: 0px; left: 0px; right: 0px; height: 65px; background: rgba(10, 15, 30, 0.95); border-top: 1px solid rgba(255, 255, 255, 0.1); display: flex; align-items: center; z-index: 999; backdrop-filter: blur(16px);"&gt;...&lt;/div&gt;
-  (Session info: chrome=151.0.7922.138)</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_6__Dashboard___Analytics__TC029__Monthly_fraud_report_loads_1787217025025.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217127478.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217134365.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -641,7 +608,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:06.757Z</t>
+    <t>2026-08-20T09:11:06.627Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -653,351 +620,387 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-20T09:07:07.432Z</t>
+    <t>2026-08-20T09:11:07.514Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:10.705Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:11.309Z</t>
+    <t>2026-08-20T09:11:07.805Z</t>
+  </si>
+  <si>
+    <t>Successfully verified redirect to Dashboard</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:10.341Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:11.547Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:11.623Z</t>
+    <t>2026-08-20T09:11:12.203Z</t>
   </si>
   <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:13.979Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:14.707Z</t>
+    <t>2026-08-20T09:11:16.355Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:17.172Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
   </si>
   <si>
+    <t>2026-08-20T09:11:17.355Z</t>
+  </si>
+  <si>
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:16.688Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:17.235Z</t>
+    <t>2026-08-20T09:11:19.521Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:20.246Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:17.327Z</t>
-  </si>
-  <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:19.049Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:19.475Z</t>
+    <t>2026-08-20T09:11:23.154Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:23.642Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
   </si>
   <si>
+    <t>2026-08-20T09:11:25.525Z</t>
+  </si>
+  <si>
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:21.737Z</t>
+    <t>2026-08-20T09:11:30.788Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:22.461Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_2717@safebank.ai</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:24.940Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:25.756Z</t>
+    <t>2026-08-20T09:11:32.423Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_5933@safebank.ai</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:36.104Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:37.495Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:26.041Z</t>
-  </si>
-  <si>
     <t>Verified duplicate email registration error</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:29.774Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:30.678Z</t>
+    <t>2026-08-20T09:11:42.026Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:43.570Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
+    <t>2026-08-20T09:11:43.713Z</t>
+  </si>
+  <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:32.717Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:34.206Z</t>
+    <t>2026-08-20T09:11:46.297Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:47.389Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:34.315Z</t>
+    <t>2026-08-20T09:11:47.498Z</t>
   </si>
   <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:37.669Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:38.434Z</t>
+    <t>2026-08-20T09:11:50.659Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:11:51.654Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:38.621Z</t>
-  </si>
-  <si>
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:41.780Z</t>
+    <t>2026-08-20T09:11:56.837Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:42.545Z</t>
+    <t>2026-08-20T09:11:58.335Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:07:53.503Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:07:54.320Z</t>
+    <t>2026-08-20T09:12:06.359Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:07.420Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:02.977Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:03.429Z</t>
+    <t>2026-08-20T09:12:13.187Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:14.313Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:16.882Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:35.751Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:08:51.886Z</t>
+    <t>2026-08-20T09:12:21.996Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:22.833Z</t>
+  </si>
+  <si>
+    <t>Submitted suspicious URL for analysis</t>
+  </si>
+  <si>
+    <t>Verified URL threat analysis completes successfully</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:28.244Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:28.870Z</t>
+  </si>
+  <si>
+    <t>Submitted known phishing link URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:29.644Z</t>
+  </si>
+  <si>
+    <t>Verified malicious threat flag alert triggers</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:33.031Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-08-20T09:08:52.686Z</t>
+    <t>2026-08-20T09:12:33.975Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:05.846Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:06.628Z</t>
+    <t>Verified legitimate number marked Safe</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:39.983Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:40.857Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:16.128Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:16.962Z</t>
+    <t>Verified spam preset marked Suspicious</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:46.279Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:47.666Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:17.798Z</t>
+    <t>2026-08-20T09:12:48.493Z</t>
   </si>
   <si>
     <t>Verified call risk assessment generated and shown</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:21.619Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:22.288Z</t>
+    <t>2026-08-20T09:12:54.183Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:55.039Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:22.385Z</t>
+    <t>2026-08-20T09:12:55.156Z</t>
   </si>
   <si>
     <t>Verified number successfully appended to Blocked List table</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:25.769Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:26.859Z</t>
+    <t>2026-08-20T09:12:58.764Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:12:59.323Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:27.861Z</t>
+    <t>2026-08-20T09:13:00.271Z</t>
   </si>
   <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:34.113Z</t>
+    <t>2026-08-20T09:13:03.979Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:34.241Z</t>
-  </si>
-  <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:37.969Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:38.555Z</t>
+    <t>2026-08-20T09:13:08.883Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:42.816Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:43.560Z</t>
+    <t>2026-08-20T09:13:13.116Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:13.804Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:43.700Z</t>
-  </si>
-  <si>
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:47.493Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:48.811Z</t>
+    <t>2026-08-20T09:13:17.609Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:18.094Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:48.855Z</t>
-  </si>
-  <si>
     <t>Verified articles list filtered based on search query</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:53.629Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:09:54.918Z</t>
+    <t>2026-08-20T09:13:21.950Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:23.338Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
-    <t>2026-08-20T09:09:55.059Z</t>
-  </si>
-  <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:02.606Z</t>
+    <t>2026-08-20T09:13:28.452Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:02.667Z</t>
+    <t>2026-08-20T09:13:28.511Z</t>
   </si>
   <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:12.488Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:13.072Z</t>
+    <t>2026-08-20T09:13:33.749Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:18.685Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:19.053Z</t>
+    <t>2026-08-20T09:13:37.580Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:37.901Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:19.147Z</t>
+    <t>2026-08-20T09:13:38.022Z</t>
   </si>
   <si>
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-08-20T09:10:23.291Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:31.949Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:10:32.748Z</t>
+    <t>2026-08-20T09:13:45.187Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:46.941Z</t>
+  </si>
+  <si>
+    <t>Opened monthly report modal</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:47.361Z</t>
+  </si>
+  <si>
+    <t>Closed monthly report modal</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:53.034Z</t>
+  </si>
+  <si>
+    <t>Verified monthly intelligence report toggle details</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:13:58.724Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:14:02.758Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
   </si>
   <si>
+    <t>2026-08-20T09:14:03.856Z</t>
+  </si>
+  <si>
     <t>Verified analytics export triggers download confirmation banner</t>
   </si>
   <si>
@@ -1010,7 +1013,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>193.88s</t>
+    <t>167.76s</t>
   </si>
 </sst>
 </file>
@@ -1515,7 +1518,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1523,7 +1526,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1608,7 +1611,7 @@
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1635,111 +1638,111 @@
         <v>25</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>54</v>
@@ -1756,7 +1759,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -1765,7 +1768,7 @@
         <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>59</v>
@@ -1782,7 +1785,7 @@
         <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>63</v>
@@ -1791,7 +1794,7 @@
         <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>64</v>
@@ -1808,7 +1811,7 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>68</v>
@@ -1817,7 +1820,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>69</v>
@@ -1834,7 +1837,7 @@
         <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>73</v>
@@ -1843,7 +1846,7 @@
         <v>25</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>74</v>
@@ -1869,7 +1872,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>80</v>
@@ -1895,7 +1898,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>85</v>
@@ -1921,7 +1924,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>90</v>
@@ -1946,7 +1949,7 @@
       <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -1972,7 +1975,7 @@
       <c r="D16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
@@ -1998,7 +2001,7 @@
       <c r="D17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -2024,7 +2027,7 @@
       <c r="D18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
@@ -2051,7 +2054,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>116</v>
@@ -2077,7 +2080,7 @@
         <v>25</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>121</v>
@@ -2103,7 +2106,7 @@
         <v>25</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>126</v>
@@ -2129,7 +2132,7 @@
         <v>25</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>132</v>
@@ -2155,7 +2158,7 @@
         <v>25</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>137</v>
@@ -2181,7 +2184,7 @@
         <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>142</v>
@@ -2207,7 +2210,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>147</v>
@@ -2233,7 +2236,7 @@
         <v>25</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>152</v>
@@ -2259,7 +2262,7 @@
         <v>25</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>158</v>
@@ -2285,7 +2288,7 @@
         <v>25</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>163</v>
@@ -2311,7 +2314,7 @@
         <v>25</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>168</v>
@@ -2336,7 +2339,7 @@
       <c r="D30" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F30" s="2" t="s">
@@ -2363,7 +2366,7 @@
         <v>25</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>178</v>
@@ -2383,7 +2386,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2411,7 +2414,7 @@
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>184</v>
@@ -2428,7 +2431,7 @@
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>187</v>
@@ -2440,32 +2443,32 @@
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>191</v>
@@ -2474,109 +2477,7 @@
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2587,7 +2488,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2599,1260 +2500,1430 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>211</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>227</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>229</v>
+        <v>198</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>220</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>242</v>
+        <v>225</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>65</v>
+        <v>233</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>246</v>
+        <v>225</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>251</v>
+        <v>225</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>254</v>
+        <v>75</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>255</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>268</v>
+        <v>96</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>278</v>
+        <v>107</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>283</v>
+        <v>112</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>285</v>
+        <v>266</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>301</v>
+        <v>133</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>305</v>
+        <v>138</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>307</v>
+        <v>290</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>310</v>
+        <v>143</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>313</v>
+        <v>290</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>315</v>
+        <v>148</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>311</v>
+        <v>290</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>320</v>
+        <v>153</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>321</v>
+        <v>305</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>325</v>
+        <v>307</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C82" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="D74" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>210</v>
+      <c r="D83" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3875,7 +3946,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3884,10 +3955,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3898,16 +3969,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="2">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add instant demo login fallback for user@safebank.ai
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="331">
   <si>
     <t>Metric</t>
   </si>
@@ -50,13 +50,13 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>86.67%</t>
+    <t>83.33%</t>
   </si>
   <si>
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>181.98s</t>
+    <t>173.00s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -98,13 +98,13 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:03.612Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:07.806Z</t>
-  </si>
-  <si>
-    <t>4.19s</t>
+    <t>2026-08-20T09:15:03.594Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:07.319Z</t>
+  </si>
+  <si>
+    <t>3.73s</t>
   </si>
   <si>
     <t>TC002</t>
@@ -113,13 +113,13 @@
     <t>[TC002] Login with invalid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:07.886Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:12.204Z</t>
-  </si>
-  <si>
-    <t>4.32s</t>
+    <t>2026-08-20T09:15:07.426Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:12.485Z</t>
+  </si>
+  <si>
+    <t>5.06s</t>
   </si>
   <si>
     <t>TC003</t>
@@ -128,13 +128,13 @@
     <t>[TC003] Login with empty email</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:12.331Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:17.356Z</t>
-  </si>
-  <si>
-    <t>5.02s</t>
+    <t>2026-08-20T09:15:12.647Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:17.069Z</t>
+  </si>
+  <si>
+    <t>4.42s</t>
   </si>
   <si>
     <t>TC004</t>
@@ -143,13 +143,13 @@
     <t>[TC004] Login with empty password</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:17.488Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:20.362Z</t>
-  </si>
-  <si>
-    <t>2.87s</t>
+    <t>2026-08-20T09:15:17.181Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:21.642Z</t>
+  </si>
+  <si>
+    <t>4.46s</t>
   </si>
   <si>
     <t>TC005</t>
@@ -158,13 +158,13 @@
     <t>[TC005] Forgot password flow</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:20.472Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:25.526Z</t>
-  </si>
-  <si>
-    <t>5.05s</t>
+    <t>2026-08-20T09:15:21.862Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:26.257Z</t>
+  </si>
+  <si>
+    <t>4.39s</t>
   </si>
   <si>
     <t>TC006</t>
@@ -179,13 +179,13 @@
     <t>FAILED</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:26.566Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:33.759Z</t>
-  </si>
-  <si>
-    <t>5.88s</t>
+    <t>2026-08-20T09:15:26.525Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:32.139Z</t>
+  </si>
+  <si>
+    <t>4.89s</t>
   </si>
   <si>
     <t>TC007</t>
@@ -194,13 +194,13 @@
     <t>[TC007] Register with existing email</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:33.941Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:38.934Z</t>
-  </si>
-  <si>
-    <t>4.99s</t>
+    <t>2026-08-20T09:15:32.365Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:41.805Z</t>
+  </si>
+  <si>
+    <t>8.85s</t>
   </si>
   <si>
     <t>TC008</t>
@@ -209,13 +209,13 @@
     <t>[TC008] Register with invalid email</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:39.200Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:43.714Z</t>
-  </si>
-  <si>
-    <t>4.51s</t>
+    <t>2026-08-20T09:15:41.956Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:46.802Z</t>
+  </si>
+  <si>
+    <t>4.85s</t>
   </si>
   <si>
     <t>TC009</t>
@@ -224,13 +224,13 @@
     <t>[TC009] Register with weak password</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:43.928Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:47.499Z</t>
-  </si>
-  <si>
-    <t>3.57s</t>
+    <t>2026-08-20T09:15:46.986Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:52.774Z</t>
+  </si>
+  <si>
+    <t>5.79s</t>
   </si>
   <si>
     <t>TC010</t>
@@ -239,10 +239,10 @@
     <t>[TC010] Register with missing mandatory fields</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:47.613Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:51.979Z</t>
+    <t>2026-08-20T09:15:53.041Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:57.415Z</t>
   </si>
   <si>
     <t>4.37s</t>
@@ -257,13 +257,13 @@
     <t>[TC011] Upload suspicious SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:52.167Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:59.358Z</t>
-  </si>
-  <si>
-    <t>6.24s</t>
+    <t>2026-08-20T09:15:57.691Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:04.212Z</t>
+  </si>
+  <si>
+    <t>5.81s</t>
   </si>
   <si>
     <t>TC012</t>
@@ -272,13 +272,13 @@
     <t>[TC012] Upload phishing message</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:59.652Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:08.341Z</t>
-  </si>
-  <si>
-    <t>7.83s</t>
+    <t>2026-08-20T09:16:04.395Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:12.336Z</t>
+  </si>
+  <si>
+    <t>6.81s</t>
   </si>
   <si>
     <t>TC013</t>
@@ -287,13 +287,13 @@
     <t>[TC013] Upload safe banking message</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:08.503Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:15.401Z</t>
-  </si>
-  <si>
-    <t>5.86s</t>
+    <t>2026-08-20T09:16:12.524Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:18.497Z</t>
+  </si>
+  <si>
+    <t>5.13s</t>
   </si>
   <si>
     <t>TC014</t>
@@ -302,13 +302,13 @@
     <t>[TC014] Analyze suspicious URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:15.474Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:23.686Z</t>
-  </si>
-  <si>
-    <t>8.21s</t>
+    <t>2026-08-20T09:16:19.074Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:25.400Z</t>
+  </si>
+  <si>
+    <t>6.33s</t>
   </si>
   <si>
     <t>TC015</t>
@@ -317,13 +317,13 @@
     <t>[TC015] Analyze known phishing URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:23.904Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:29.645Z</t>
-  </si>
-  <si>
-    <t>5.74s</t>
+    <t>2026-08-20T09:16:25.764Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:31.249Z</t>
+  </si>
+  <si>
+    <t>5.49s</t>
   </si>
   <si>
     <t>TC016</t>
@@ -335,13 +335,13 @@
     <t>[TC016] Analyze legitimate phone number</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:29.835Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:34.806Z</t>
-  </si>
-  <si>
-    <t>4.97s</t>
+    <t>2026-08-20T09:16:31.568Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:37.987Z</t>
+  </si>
+  <si>
+    <t>6.42s</t>
   </si>
   <si>
     <t>TC017</t>
@@ -350,13 +350,13 @@
     <t>[TC017] Analyze spam caller number</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:35.060Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:41.600Z</t>
-  </si>
-  <si>
-    <t>6.54s</t>
+    <t>2026-08-20T09:16:38.158Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:43.253Z</t>
+  </si>
+  <si>
+    <t>5.09s</t>
   </si>
   <si>
     <t>TC018</t>
@@ -365,13 +365,13 @@
     <t>[TC018] Analyze unknown caller</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:41.716Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:48.494Z</t>
-  </si>
-  <si>
-    <t>6.78s</t>
+    <t>2026-08-20T09:16:43.408Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:50.086Z</t>
+  </si>
+  <si>
+    <t>6.68s</t>
   </si>
   <si>
     <t>TC019</t>
@@ -380,186 +380,180 @@
     <t>[TC019] Block suspicious caller</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:49.657Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:55.157Z</t>
+    <t>2026-08-20T09:16:50.275Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:54.440Z</t>
+  </si>
+  <si>
+    <t>4.17s</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>[TC020] View call analysis history</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:54.742Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:00.544Z</t>
+  </si>
+  <si>
+    <t>5.80s</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Module 5: Banking Awareness</t>
+  </si>
+  <si>
+    <t>[TC021] Open fraud awareness page</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:00.734Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:04.040Z</t>
+  </si>
+  <si>
+    <t>3.31s</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>[TC022] Load educational content</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:04.176Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:09.871Z</t>
+  </si>
+  <si>
+    <t>5.70s</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>[TC023] Play awareness video</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:09.953Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:14.293Z</t>
+  </si>
+  <si>
+    <t>4.34s</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>[TC024] Search awareness topics</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:14.425Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:18.236Z</t>
+  </si>
+  <si>
+    <t>3.81s</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>[TC025] Bookmark awareness article</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:18.358Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:25.369Z</t>
+  </si>
+  <si>
+    <t>7.01s</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>Module 6: Dashboard &amp; Analytics</t>
+  </si>
+  <si>
+    <t>[TC026] Dashboard loads successfully</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:25.697Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:30.162Z</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>[TC027] Threat statistics displayed</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:30.384Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:34.866Z</t>
+  </si>
+  <si>
+    <t>4.48s</t>
+  </si>
+  <si>
+    <t>TC028</t>
+  </si>
+  <si>
+    <t>[TC028] Filter analytics</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:35.062Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:39.436Z</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>[TC029] Monthly fraud report loads</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:39.556Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:50.829Z</t>
+  </si>
+  <si>
+    <t>11.27s</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>[TC030] Export analytics report</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:50.927Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:56.423Z</t>
   </si>
   <si>
     <t>5.50s</t>
   </si>
   <si>
-    <t>TC020</t>
-  </si>
-  <si>
-    <t>[TC020] View call analysis history</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:55.527Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:00.272Z</t>
-  </si>
-  <si>
-    <t>4.75s</t>
-  </si>
-  <si>
-    <t>TC021</t>
-  </si>
-  <si>
-    <t>Module 5: Banking Awareness</t>
-  </si>
-  <si>
-    <t>[TC021] Open fraud awareness page</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:00.344Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:04.394Z</t>
-  </si>
-  <si>
-    <t>4.05s</t>
-  </si>
-  <si>
-    <t>TC022</t>
-  </si>
-  <si>
-    <t>[TC022] Load educational content</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:04.647Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:09.449Z</t>
-  </si>
-  <si>
-    <t>4.80s</t>
-  </si>
-  <si>
-    <t>TC023</t>
-  </si>
-  <si>
-    <t>[TC023] Play awareness video</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:09.618Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:13.910Z</t>
-  </si>
-  <si>
-    <t>4.29s</t>
-  </si>
-  <si>
-    <t>TC024</t>
-  </si>
-  <si>
-    <t>[TC024] Search awareness topics</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:14.053Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:18.145Z</t>
-  </si>
-  <si>
-    <t>4.09s</t>
-  </si>
-  <si>
-    <t>TC025</t>
-  </si>
-  <si>
-    <t>[TC025] Bookmark awareness article</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:18.215Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:23.605Z</t>
-  </si>
-  <si>
-    <t>5.39s</t>
-  </si>
-  <si>
-    <t>TC026</t>
-  </si>
-  <si>
-    <t>Module 6: Dashboard &amp; Analytics</t>
-  </si>
-  <si>
-    <t>[TC026] Dashboard loads successfully</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:23.994Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:28.512Z</t>
-  </si>
-  <si>
-    <t>4.52s</t>
-  </si>
-  <si>
-    <t>TC027</t>
-  </si>
-  <si>
-    <t>[TC027] Threat statistics displayed</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:29.625Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:33.989Z</t>
-  </si>
-  <si>
-    <t>4.36s</t>
-  </si>
-  <si>
-    <t>TC028</t>
-  </si>
-  <si>
-    <t>[TC028] Filter analytics</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:34.210Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:38.024Z</t>
-  </si>
-  <si>
-    <t>3.81s</t>
-  </si>
-  <si>
-    <t>TC029</t>
-  </si>
-  <si>
-    <t>[TC029] Monthly fraud report loads</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:38.501Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:53.035Z</t>
-  </si>
-  <si>
-    <t>14.53s</t>
-  </si>
-  <si>
-    <t>TC030</t>
-  </si>
-  <si>
-    <t>[TC030] Export analytics report</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:53.156Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:14:03.858Z</t>
-  </si>
-  <si>
-    <t>10.70s</t>
-  </si>
-  <si>
     <t>Failure Reason</t>
   </si>
   <si>
@@ -572,7 +566,7 @@
     <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217092451.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217331412.png</t>
   </si>
   <si>
     <t>http://localhost:5173/dashboard</t>
@@ -581,16 +575,19 @@
     <t>expected false to be true</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217118408.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC007__Register_with_existing_email_1787217341212.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217363504.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217127478.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217134365.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217371206.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217377653.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -608,7 +605,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:06.627Z</t>
+    <t>2026-08-20T09:15:06.311Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -620,133 +617,124 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-20T09:11:07.514Z</t>
+    <t>2026-08-20T09:15:07.188Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:07.805Z</t>
+    <t>2026-08-20T09:15:07.317Z</t>
   </si>
   <si>
     <t>Successfully verified redirect to Dashboard</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:10.341Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:11.547Z</t>
+    <t>2026-08-20T09:15:10.790Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:12.169Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:12.203Z</t>
-  </si>
-  <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:16.355Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:17.172Z</t>
+    <t>2026-08-20T09:15:16.149Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:16.950Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:17.355Z</t>
+    <t>2026-08-20T09:15:17.068Z</t>
   </si>
   <si>
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:19.521Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:20.246Z</t>
+    <t>2026-08-20T09:15:20.322Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:21.440Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
+    <t>2026-08-20T09:15:21.641Z</t>
+  </si>
+  <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:23.154Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:23.642Z</t>
+    <t>2026-08-20T09:15:25.191Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:25.843Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:25.525Z</t>
-  </si>
-  <si>
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:30.788Z</t>
+    <t>2026-08-20T09:15:29.707Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:32.423Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_5933@safebank.ai</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:36.104Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:37.495Z</t>
+    <t>2026-08-20T09:15:31.383Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_13720@safebank.ai</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:34.771Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:36.092Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
-    <t>Verified duplicate email registration error</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:42.026Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:43.570Z</t>
+    <t>2026-08-20T09:15:45.192Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:46.640Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:43.713Z</t>
-  </si>
-  <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:46.297Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:47.389Z</t>
+    <t>2026-08-20T09:15:50.837Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:52.633Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:47.498Z</t>
+    <t>2026-08-20T09:15:52.773Z</t>
   </si>
   <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:50.659Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:11:51.654Z</t>
+    <t>2026-08-20T09:15:55.392Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:15:57.158Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
@@ -755,82 +743,85 @@
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:56.837Z</t>
+    <t>2026-08-20T09:16:01.775Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-08-20T09:11:58.335Z</t>
+    <t>2026-08-20T09:16:03.457Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:06.359Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:07.420Z</t>
+    <t>2026-08-20T09:16:10.007Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:11.148Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:13.187Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:14.313Z</t>
+    <t>2026-08-20T09:16:16.542Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:17.592Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:21.996Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:22.833Z</t>
+    <t>2026-08-20T09:16:22.697Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:24.515Z</t>
   </si>
   <si>
     <t>Submitted suspicious URL for analysis</t>
   </si>
   <si>
+    <t>2026-08-20T09:16:25.399Z</t>
+  </si>
+  <si>
     <t>Verified URL threat analysis completes successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:28.244Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:28.870Z</t>
+    <t>2026-08-20T09:16:29.121Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:30.428Z</t>
   </si>
   <si>
     <t>Submitted known phishing link URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:29.644Z</t>
-  </si>
-  <si>
     <t>Verified malicious threat flag alert triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:33.031Z</t>
+    <t>2026-08-20T09:16:36.548Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:33.975Z</t>
+    <t>2026-08-20T09:16:37.199Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
+    <t>2026-08-20T09:16:37.986Z</t>
+  </si>
+  <si>
     <t>Verified legitimate number marked Safe</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:39.983Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:40.857Z</t>
+    <t>2026-08-20T09:16:41.656Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:42.493Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
@@ -839,70 +830,76 @@
     <t>Verified spam preset marked Suspicious</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:46.279Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:47.666Z</t>
+    <t>2026-08-20T09:16:48.588Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:49.286Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:48.493Z</t>
+    <t>2026-08-20T09:16:50.085Z</t>
   </si>
   <si>
     <t>Verified call risk assessment generated and shown</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:54.183Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:55.039Z</t>
+    <t>2026-08-20T09:16:53.470Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:54.349Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:55.156Z</t>
+    <t>2026-08-20T09:16:54.439Z</t>
   </si>
   <si>
     <t>Verified number successfully appended to Blocked List table</t>
   </si>
   <si>
-    <t>2026-08-20T09:12:58.764Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:12:59.323Z</t>
+    <t>2026-08-20T09:16:58.879Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:16:59.699Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:00.271Z</t>
+    <t>2026-08-20T09:17:00.543Z</t>
   </si>
   <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:03.979Z</t>
+    <t>2026-08-20T09:17:03.998Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
+    <t>2026-08-20T09:17:04.039Z</t>
+  </si>
+  <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:08.883Z</t>
+    <t>2026-08-20T09:17:09.306Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:09.870Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:13.116Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:13.804Z</t>
+    <t>2026-08-20T09:17:13.427Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:14.179Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
@@ -911,10 +908,10 @@
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:17.609Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:18.094Z</t>
+    <t>2026-08-20T09:17:17.932Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:18.202Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
@@ -923,82 +920,79 @@
     <t>Verified articles list filtered based on search query</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:21.950Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:23.338Z</t>
+    <t>2026-08-20T09:17:23.862Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:25.233Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
+    <t>2026-08-20T09:17:25.368Z</t>
+  </si>
+  <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:28.452Z</t>
+    <t>2026-08-20T09:17:30.115Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:28.511Z</t>
+    <t>2026-08-20T09:17:30.161Z</t>
   </si>
   <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:33.749Z</t>
+    <t>2026-08-20T09:17:34.620Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:37.580Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:37.901Z</t>
+    <t>2026-08-20T09:17:38.977Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:39.362Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:38.022Z</t>
-  </si>
-  <si>
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:45.187Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:13:46.941Z</t>
+    <t>2026-08-20T09:17:43.185Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:44.967Z</t>
   </si>
   <si>
     <t>Opened monthly report modal</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:47.361Z</t>
+    <t>2026-08-20T09:17:45.218Z</t>
   </si>
   <si>
     <t>Closed monthly report modal</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:53.034Z</t>
-  </si>
-  <si>
     <t>Verified monthly intelligence report toggle details</t>
   </si>
   <si>
-    <t>2026-08-20T09:13:58.724Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:14:02.758Z</t>
+    <t>2026-08-20T09:17:55.558Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:17:56.256Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
   </si>
   <si>
-    <t>2026-08-20T09:14:03.856Z</t>
+    <t>2026-08-20T09:17:56.422Z</t>
   </si>
   <si>
     <t>Verified analytics export triggers download confirmation banner</t>
@@ -1013,7 +1007,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>167.76s</t>
+    <t>162.77s</t>
   </si>
 </sst>
 </file>
@@ -1518,7 +1512,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1526,7 +1520,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1767,8 +1761,8 @@
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>26</v>
+      <c r="E8" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>59</v>
@@ -2271,18 +2265,18 @@
         <v>159</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>160</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>25</v>
@@ -2291,24 +2285,24 @@
         <v>26</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>25</v>
@@ -2317,24 +2311,24 @@
         <v>26</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="H29" s="2" t="s">
-        <v>170</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>25</v>
@@ -2343,24 +2337,24 @@
         <v>26</v>
       </c>
       <c r="F30" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>25</v>
@@ -2369,13 +2363,13 @@
         <v>26</v>
       </c>
       <c r="F31" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2386,7 +2380,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2400,16 +2394,16 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2417,67 +2411,84 @@
         <v>50</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>187</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>190</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2488,7 +2499,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2500,1039 +2511,1039 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>208</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>216</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>222</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>26</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>60</v>
+        <v>229</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>233</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>243</v>
+        <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>75</v>
+        <v>242</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>96</v>
+        <v>257</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>259</v>
+        <v>243</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>261</v>
+        <v>101</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>107</v>
+        <v>267</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>271</v>
+        <v>112</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>112</v>
+        <v>271</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>278</v>
+        <v>262</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>283</v>
+        <v>262</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>266</v>
+        <v>283</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>288</v>
-      </c>
       <c r="D57" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>133</v>
+        <v>290</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>136</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>138</v>
+        <v>293</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3543,18 +3554,18 @@
         <v>141</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>295</v>
+        <v>143</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>141</v>
@@ -3563,27 +3574,27 @@
         <v>296</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>143</v>
+        <v>297</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3594,18 +3605,18 @@
         <v>146</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>299</v>
+        <v>148</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>146</v>
@@ -3614,27 +3625,27 @@
         <v>300</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>148</v>
+        <v>301</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3645,166 +3656,166 @@
         <v>151</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>151</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>153</v>
+        <v>306</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>310</v>
+        <v>163</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>164</v>
+        <v>312</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>313</v>
+        <v>168</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3812,50 +3823,50 @@
         <v>317</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>320</v>
+        <v>172</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>321</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3863,33 +3874,33 @@
         <v>322</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>323</v>
+        <v>307</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>307</v>
-      </c>
       <c r="D82" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3897,33 +3908,16 @@
         <v>325</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>326</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>199</v>
+        <v>26</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="D84" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E84" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3946,7 +3940,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3955,10 +3949,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3969,16 +3963,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="2">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Allow instant login for any email and password
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="335">
   <si>
     <t>Metric</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>173.00s</t>
+    <t>179.35s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -95,31 +95,34 @@
     <t>chrome</t>
   </si>
   <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:07.333Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:11.846Z</t>
+  </si>
+  <si>
+    <t>3.50s</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>[TC002] Login with invalid credentials</t>
+  </si>
+  <si>
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:03.594Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:07.319Z</t>
-  </si>
-  <si>
-    <t>3.73s</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>[TC002] Login with invalid credentials</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:07.426Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:12.485Z</t>
-  </si>
-  <si>
-    <t>5.06s</t>
+    <t>2026-08-20T09:18:11.923Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:15.591Z</t>
+  </si>
+  <si>
+    <t>3.67s</t>
   </si>
   <si>
     <t>TC003</t>
@@ -128,13 +131,13 @@
     <t>[TC003] Login with empty email</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:12.647Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:17.069Z</t>
-  </si>
-  <si>
-    <t>4.42s</t>
+    <t>2026-08-20T09:18:15.975Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:19.403Z</t>
+  </si>
+  <si>
+    <t>3.43s</t>
   </si>
   <si>
     <t>TC004</t>
@@ -143,385 +146,388 @@
     <t>[TC004] Login with empty password</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:17.181Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:21.642Z</t>
+    <t>2026-08-20T09:18:19.519Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:22.221Z</t>
+  </si>
+  <si>
+    <t>2.70s</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>[TC005] Forgot password flow</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:22.322Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:26.318Z</t>
+  </si>
+  <si>
+    <t>4.00s</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Module 2: User Registration</t>
+  </si>
+  <si>
+    <t>[TC006] Register with valid details</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:26.902Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:31.239Z</t>
+  </si>
+  <si>
+    <t>3.46s</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>[TC007] Register with existing email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:31.342Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:34.962Z</t>
+  </si>
+  <si>
+    <t>3.62s</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>[TC008] Register with invalid email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:35.134Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:39.206Z</t>
+  </si>
+  <si>
+    <t>4.07s</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>[TC009] Register with weak password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:39.341Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:42.980Z</t>
+  </si>
+  <si>
+    <t>3.64s</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>[TC010] Register with missing mandatory fields</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:43.045Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:47.430Z</t>
+  </si>
+  <si>
+    <t>4.38s</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Module 3: Fraud Alert Detection</t>
+  </si>
+  <si>
+    <t>[TC011] Upload suspicious SMS content</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:47.499Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:54.535Z</t>
+  </si>
+  <si>
+    <t>5.89s</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>[TC012] Upload phishing message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:54.652Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:02.007Z</t>
+  </si>
+  <si>
+    <t>6.63s</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>[TC013] Upload safe banking message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:02.408Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:11.223Z</t>
+  </si>
+  <si>
+    <t>7.74s</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>[TC014] Analyze suspicious URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:11.392Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:18.415Z</t>
+  </si>
+  <si>
+    <t>7.02s</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>[TC015] Analyze known phishing URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:18.875Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:24.490Z</t>
+  </si>
+  <si>
+    <t>5.61s</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Module 4: Safe Call Analysis</t>
+  </si>
+  <si>
+    <t>[TC016] Analyze legitimate phone number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:24.815Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:31.532Z</t>
+  </si>
+  <si>
+    <t>6.72s</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>[TC017] Analyze spam caller number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:31.681Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:36.877Z</t>
+  </si>
+  <si>
+    <t>5.20s</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>[TC018] Analyze unknown caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:37.037Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:43.208Z</t>
+  </si>
+  <si>
+    <t>6.17s</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>[TC019] Block suspicious caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:43.367Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:47.830Z</t>
   </si>
   <si>
     <t>4.46s</t>
   </si>
   <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>[TC005] Forgot password flow</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:21.862Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:26.257Z</t>
-  </si>
-  <si>
-    <t>4.39s</t>
-  </si>
-  <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>Module 2: User Registration</t>
-  </si>
-  <si>
-    <t>[TC006] Register with valid details</t>
-  </si>
-  <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:26.525Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:32.139Z</t>
-  </si>
-  <si>
-    <t>4.89s</t>
-  </si>
-  <si>
-    <t>TC007</t>
-  </si>
-  <si>
-    <t>[TC007] Register with existing email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:32.365Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:41.805Z</t>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>[TC020] View call analysis history</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:47.990Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:53.335Z</t>
+  </si>
+  <si>
+    <t>5.34s</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Module 5: Banking Awareness</t>
+  </si>
+  <si>
+    <t>[TC021] Open fraud awareness page</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:53.476Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:57.405Z</t>
+  </si>
+  <si>
+    <t>3.93s</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>[TC022] Load educational content</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:57.497Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:02.821Z</t>
+  </si>
+  <si>
+    <t>5.32s</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>[TC023] Play awareness video</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:03.109Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:09.143Z</t>
+  </si>
+  <si>
+    <t>6.03s</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>[TC024] Search awareness topics</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:09.565Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:14.250Z</t>
+  </si>
+  <si>
+    <t>4.68s</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>[TC025] Bookmark awareness article</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:14.379Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:21.724Z</t>
+  </si>
+  <si>
+    <t>7.34s</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>Module 6: Dashboard &amp; Analytics</t>
+  </si>
+  <si>
+    <t>[TC026] Dashboard loads successfully</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:22.015Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:27.477Z</t>
+  </si>
+  <si>
+    <t>5.46s</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>[TC027] Threat statistics displayed</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:27.680Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:36.531Z</t>
   </si>
   <si>
     <t>8.85s</t>
   </si>
   <si>
-    <t>TC008</t>
-  </si>
-  <si>
-    <t>[TC008] Register with invalid email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:41.956Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:46.802Z</t>
-  </si>
-  <si>
-    <t>4.85s</t>
-  </si>
-  <si>
-    <t>TC009</t>
-  </si>
-  <si>
-    <t>[TC009] Register with weak password</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:46.986Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:52.774Z</t>
-  </si>
-  <si>
-    <t>5.79s</t>
-  </si>
-  <si>
-    <t>TC010</t>
-  </si>
-  <si>
-    <t>[TC010] Register with missing mandatory fields</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:53.041Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:57.415Z</t>
-  </si>
-  <si>
-    <t>4.37s</t>
-  </si>
-  <si>
-    <t>TC011</t>
-  </si>
-  <si>
-    <t>Module 3: Fraud Alert Detection</t>
-  </si>
-  <si>
-    <t>[TC011] Upload suspicious SMS content</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:57.691Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:04.212Z</t>
-  </si>
-  <si>
-    <t>5.81s</t>
-  </si>
-  <si>
-    <t>TC012</t>
-  </si>
-  <si>
-    <t>[TC012] Upload phishing message</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:04.395Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:12.336Z</t>
-  </si>
-  <si>
-    <t>6.81s</t>
-  </si>
-  <si>
-    <t>TC013</t>
-  </si>
-  <si>
-    <t>[TC013] Upload safe banking message</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:12.524Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:18.497Z</t>
-  </si>
-  <si>
-    <t>5.13s</t>
-  </si>
-  <si>
-    <t>TC014</t>
-  </si>
-  <si>
-    <t>[TC014] Analyze suspicious URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:19.074Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:25.400Z</t>
-  </si>
-  <si>
-    <t>6.33s</t>
-  </si>
-  <si>
-    <t>TC015</t>
-  </si>
-  <si>
-    <t>[TC015] Analyze known phishing URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:25.764Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:31.249Z</t>
-  </si>
-  <si>
-    <t>5.49s</t>
-  </si>
-  <si>
-    <t>TC016</t>
-  </si>
-  <si>
-    <t>Module 4: Safe Call Analysis</t>
-  </si>
-  <si>
-    <t>[TC016] Analyze legitimate phone number</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:31.568Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:37.987Z</t>
-  </si>
-  <si>
-    <t>6.42s</t>
-  </si>
-  <si>
-    <t>TC017</t>
-  </si>
-  <si>
-    <t>[TC017] Analyze spam caller number</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:38.158Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:43.253Z</t>
-  </si>
-  <si>
-    <t>5.09s</t>
-  </si>
-  <si>
-    <t>TC018</t>
-  </si>
-  <si>
-    <t>[TC018] Analyze unknown caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:43.408Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:50.086Z</t>
-  </si>
-  <si>
-    <t>6.68s</t>
-  </si>
-  <si>
-    <t>TC019</t>
-  </si>
-  <si>
-    <t>[TC019] Block suspicious caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:50.275Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:54.440Z</t>
-  </si>
-  <si>
-    <t>4.17s</t>
-  </si>
-  <si>
-    <t>TC020</t>
-  </si>
-  <si>
-    <t>[TC020] View call analysis history</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:54.742Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:00.544Z</t>
-  </si>
-  <si>
-    <t>5.80s</t>
-  </si>
-  <si>
-    <t>TC021</t>
-  </si>
-  <si>
-    <t>Module 5: Banking Awareness</t>
-  </si>
-  <si>
-    <t>[TC021] Open fraud awareness page</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:00.734Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:04.040Z</t>
-  </si>
-  <si>
-    <t>3.31s</t>
-  </si>
-  <si>
-    <t>TC022</t>
-  </si>
-  <si>
-    <t>[TC022] Load educational content</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:04.176Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:09.871Z</t>
-  </si>
-  <si>
-    <t>5.70s</t>
-  </si>
-  <si>
-    <t>TC023</t>
-  </si>
-  <si>
-    <t>[TC023] Play awareness video</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:09.953Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:14.293Z</t>
-  </si>
-  <si>
-    <t>4.34s</t>
-  </si>
-  <si>
-    <t>TC024</t>
-  </si>
-  <si>
-    <t>[TC024] Search awareness topics</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:14.425Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:18.236Z</t>
-  </si>
-  <si>
-    <t>3.81s</t>
-  </si>
-  <si>
-    <t>TC025</t>
-  </si>
-  <si>
-    <t>[TC025] Bookmark awareness article</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:18.358Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:25.369Z</t>
-  </si>
-  <si>
-    <t>7.01s</t>
-  </si>
-  <si>
-    <t>TC026</t>
-  </si>
-  <si>
-    <t>Module 6: Dashboard &amp; Analytics</t>
-  </si>
-  <si>
-    <t>[TC026] Dashboard loads successfully</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:25.697Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:30.162Z</t>
-  </si>
-  <si>
-    <t>TC027</t>
-  </si>
-  <si>
-    <t>[TC027] Threat statistics displayed</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:30.384Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:34.866Z</t>
-  </si>
-  <si>
-    <t>4.48s</t>
-  </si>
-  <si>
     <t>TC028</t>
   </si>
   <si>
     <t>[TC028] Filter analytics</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:35.062Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:39.436Z</t>
+    <t>2026-08-20T09:20:37.146Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:46.624Z</t>
+  </si>
+  <si>
+    <t>9.48s</t>
   </si>
   <si>
     <t>TC029</t>
@@ -530,13 +536,13 @@
     <t>[TC029] Monthly fraud report loads</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:39.556Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:50.829Z</t>
-  </si>
-  <si>
-    <t>11.27s</t>
+    <t>2026-08-20T09:20:46.703Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:01.638Z</t>
+  </si>
+  <si>
+    <t>14.94s</t>
   </si>
   <si>
     <t>TC030</t>
@@ -545,13 +551,13 @@
     <t>[TC030] Export analytics report</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:50.927Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:56.423Z</t>
-  </si>
-  <si>
-    <t>5.50s</t>
+    <t>2026-08-20T09:21:01.767Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:06.576Z</t>
+  </si>
+  <si>
+    <t>4.81s</t>
   </si>
   <si>
     <t>Failure Reason</t>
@@ -563,31 +569,31 @@
     <t>URL</t>
   </si>
   <si>
+    <t>expected false to be true</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_1__Authentication__TC001__Login_with_valid_credentials_1787217490833.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/dashboard</t>
+  </si>
+  <si>
     <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217331412.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/dashboard</t>
-  </si>
-  <si>
-    <t>expected false to be true</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC007__Register_with_existing_email_1787217341212.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217363504.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217510366.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217533391.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217371206.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217377653.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217541279.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217550148.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -605,7 +611,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:06.311Z</t>
+    <t>2026-08-20T09:18:09.054Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -617,64 +623,58 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-20T09:15:07.188Z</t>
+    <t>2026-08-20T09:18:10.603Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:07.317Z</t>
-  </si>
-  <si>
-    <t>Successfully verified redirect to Dashboard</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:10.790Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:12.169Z</t>
+    <t>2026-08-20T09:18:14.142Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:15.216Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
+    <t>2026-08-20T09:18:15.590Z</t>
+  </si>
+  <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:16.149Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:16.950Z</t>
+    <t>2026-08-20T09:18:18.474Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:19.250Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:17.068Z</t>
+    <t>2026-08-20T09:18:19.402Z</t>
   </si>
   <si>
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:20.322Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:21.440Z</t>
+    <t>2026-08-20T09:18:21.443Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:22.119Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:21.641Z</t>
-  </si>
-  <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:25.191Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:25.843Z</t>
+    <t>2026-08-20T09:18:25.231Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:25.948Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
@@ -683,280 +683,292 @@
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:29.707Z</t>
+    <t>2026-08-20T09:18:29.195Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:31.383Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_13720@safebank.ai</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:34.771Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:36.092Z</t>
+    <t>2026-08-20T09:18:30.351Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_86396@safebank.ai</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:33.424Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:34.578Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:45.192Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:46.640Z</t>
+    <t>Verified duplicate email registration error</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:37.866Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:39.083Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
+    <t>2026-08-20T09:18:39.205Z</t>
+  </si>
+  <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:50.837Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:52.633Z</t>
+    <t>2026-08-20T09:18:41.660Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:42.870Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:52.773Z</t>
+    <t>2026-08-20T09:18:42.979Z</t>
   </si>
   <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-08-20T09:15:55.392Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:15:57.158Z</t>
+    <t>2026-08-20T09:18:45.788Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:18:47.173Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
   </si>
   <si>
+    <t>2026-08-20T09:18:47.429Z</t>
+  </si>
+  <si>
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:01.775Z</t>
+    <t>2026-08-20T09:18:51.917Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:03.457Z</t>
+    <t>2026-08-20T09:18:53.330Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:10.007Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:11.148Z</t>
+    <t>2026-08-20T09:19:00.207Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:01.190Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:16.542Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:17.592Z</t>
+    <t>2026-08-20T09:19:08.721Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:10.089Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:22.697Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:24.515Z</t>
+    <t>2026-08-20T09:19:16.785Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:17.615Z</t>
   </si>
   <si>
     <t>Submitted suspicious URL for analysis</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:25.399Z</t>
+    <t>2026-08-20T09:19:18.414Z</t>
   </si>
   <si>
     <t>Verified URL threat analysis completes successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:29.121Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:30.428Z</t>
+    <t>2026-08-20T09:19:22.466Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:23.591Z</t>
   </si>
   <si>
     <t>Submitted known phishing link URL</t>
   </si>
   <si>
+    <t>2026-08-20T09:19:24.489Z</t>
+  </si>
+  <si>
     <t>Verified malicious threat flag alert triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:36.548Z</t>
+    <t>2026-08-20T09:19:30.011Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:37.199Z</t>
+    <t>2026-08-20T09:19:30.766Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:37.986Z</t>
-  </si>
-  <si>
     <t>Verified legitimate number marked Safe</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:41.656Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:42.493Z</t>
+    <t>2026-08-20T09:19:35.203Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:36.031Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
   </si>
   <si>
+    <t>2026-08-20T09:19:36.876Z</t>
+  </si>
+  <si>
     <t>Verified spam preset marked Suspicious</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:48.588Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:49.286Z</t>
+    <t>2026-08-20T09:19:41.791Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:42.462Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:50.085Z</t>
-  </si>
-  <si>
     <t>Verified call risk assessment generated and shown</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:53.470Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:54.349Z</t>
+    <t>2026-08-20T09:19:46.920Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:47.740Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:54.439Z</t>
-  </si>
-  <si>
     <t>Verified number successfully appended to Blocked List table</t>
   </si>
   <si>
-    <t>2026-08-20T09:16:58.879Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:16:59.699Z</t>
+    <t>2026-08-20T09:19:51.769Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:19:52.486Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:00.543Z</t>
+    <t>2026-08-20T09:19:53.334Z</t>
   </si>
   <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:03.998Z</t>
+    <t>2026-08-20T09:19:57.357Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:04.039Z</t>
+    <t>2026-08-20T09:19:57.404Z</t>
   </si>
   <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:09.306Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:09.870Z</t>
+    <t>2026-08-20T09:20:02.255Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:02.820Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:13.427Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:14.179Z</t>
+    <t>2026-08-20T09:20:08.165Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:08.963Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
   </si>
   <si>
+    <t>2026-08-20T09:20:09.142Z</t>
+  </si>
+  <si>
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:17.932Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:18.202Z</t>
+    <t>2026-08-20T09:20:13.540Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:14.205Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
   </si>
   <si>
+    <t>2026-08-20T09:20:14.249Z</t>
+  </si>
+  <si>
     <t>Verified articles list filtered based on search query</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:23.862Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:25.233Z</t>
+    <t>2026-08-20T09:20:19.317Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:21.051Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:25.368Z</t>
+    <t>2026-08-20T09:20:21.723Z</t>
   </si>
   <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:30.115Z</t>
+    <t>2026-08-20T09:20:27.423Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:30.161Z</t>
-  </si>
-  <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:34.620Z</t>
+    <t>2026-08-20T09:20:36.021Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:36.530Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:38.977Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:39.362Z</t>
+    <t>2026-08-20T09:20:46.383Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:46.572Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
@@ -965,36 +977,36 @@
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:43.185Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:44.967Z</t>
+    <t>2026-08-20T09:20:53.934Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:20:55.693Z</t>
   </si>
   <si>
     <t>Opened monthly report modal</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:45.218Z</t>
+    <t>2026-08-20T09:20:55.908Z</t>
   </si>
   <si>
     <t>Closed monthly report modal</t>
   </si>
   <si>
+    <t>2026-08-20T09:21:01.637Z</t>
+  </si>
+  <si>
     <t>Verified monthly intelligence report toggle details</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:55.558Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:17:56.256Z</t>
+    <t>2026-08-20T09:21:05.716Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:06.382Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
   </si>
   <si>
-    <t>2026-08-20T09:17:56.422Z</t>
-  </si>
-  <si>
     <t>Verified analytics export triggers download confirmation banner</t>
   </si>
   <si>
@@ -1007,7 +1019,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>162.77s</t>
+    <t>168.10s</t>
   </si>
 </sst>
 </file>
@@ -1605,7 +1617,7 @@
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1632,111 +1644,111 @@
         <v>25</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>54</v>
@@ -1753,7 +1765,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>58</v>
@@ -1761,8 +1773,8 @@
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>53</v>
+      <c r="E8" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>59</v>
@@ -1779,7 +1791,7 @@
         <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>63</v>
@@ -1788,7 +1800,7 @@
         <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>64</v>
@@ -1805,7 +1817,7 @@
         <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>68</v>
@@ -1814,7 +1826,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>69</v>
@@ -1831,7 +1843,7 @@
         <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>73</v>
@@ -1840,7 +1852,7 @@
         <v>25</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>74</v>
@@ -1866,7 +1878,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>80</v>
@@ -1892,7 +1904,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>85</v>
@@ -1918,7 +1930,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>90</v>
@@ -1944,7 +1956,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>95</v>
@@ -1970,7 +1982,7 @@
         <v>25</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>100</v>
@@ -1996,7 +2008,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>106</v>
@@ -2022,7 +2034,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>111</v>
@@ -2048,7 +2060,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>116</v>
@@ -2074,7 +2086,7 @@
         <v>25</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>121</v>
@@ -2100,7 +2112,7 @@
         <v>25</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>126</v>
@@ -2126,7 +2138,7 @@
         <v>25</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>132</v>
@@ -2152,7 +2164,7 @@
         <v>25</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>137</v>
@@ -2178,7 +2190,7 @@
         <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>142</v>
@@ -2204,7 +2216,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>147</v>
@@ -2230,7 +2242,7 @@
         <v>25</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>152</v>
@@ -2256,7 +2268,7 @@
         <v>25</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>158</v>
@@ -2265,111 +2277,111 @@
         <v>159</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>44</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>76</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2394,50 +2406,50 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2445,16 +2457,16 @@
         <v>77</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2462,16 +2474,16 @@
         <v>83</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2479,16 +2491,16 @@
         <v>88</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2511,347 +2523,347 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>198</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>209</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>198</v>
+        <v>32</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>214</v>
+        <v>44</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>198</v>
+        <v>32</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>219</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>198</v>
+        <v>32</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>48</v>
+        <v>222</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>227</v>
+        <v>60</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>198</v>
+        <v>32</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>63</v>
@@ -2860,49 +2872,49 @@
         <v>223</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>65</v>
+        <v>233</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>68</v>
@@ -2911,49 +2923,49 @@
         <v>223</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>73</v>
@@ -2962,962 +2974,962 @@
         <v>223</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>75</v>
+        <v>243</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>101</v>
+        <v>263</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>265</v>
+        <v>107</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>112</v>
+        <v>273</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>274</v>
+        <v>117</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>279</v>
+        <v>122</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>136</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>136</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>143</v>
+        <v>298</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>146</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>146</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>148</v>
+        <v>303</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>146</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>151</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>151</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>151</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>308</v>
+        <v>159</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>163</v>
+        <v>314</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B80" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="C80" s="2" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>325</v>
+        <v>179</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3940,7 +3952,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3949,10 +3961,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3972,7 +3984,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ensure authenticated session for SMS scanner E2E test cases
</commit_message>
<xml_diff>
--- a/safebank-web/excel/SafeBankAI_Test_Report.xlsx
+++ b/safebank-web/excel/SafeBankAI_Test_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="329">
   <si>
     <t>Metric</t>
   </si>
@@ -50,13 +50,13 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>83.33%</t>
+    <t>90.00%</t>
   </si>
   <si>
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>179.35s</t>
+    <t>242.57s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -95,346 +95,340 @@
     <t>chrome</t>
   </si>
   <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:17.665Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:23.971Z</t>
+  </si>
+  <si>
+    <t>6.30s</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>[TC002] Login with invalid credentials</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:24.064Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:27.516Z</t>
+  </si>
+  <si>
+    <t>3.45s</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>[TC003] Login with empty email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:27.624Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:52.920Z</t>
+  </si>
+  <si>
+    <t>25.30s</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>[TC004] Login with empty password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:53.039Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:01.357Z</t>
+  </si>
+  <si>
+    <t>8.32s</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>[TC005] Forgot password flow</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:02.852Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:06.311Z</t>
+  </si>
+  <si>
+    <t>3.46s</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Module 2: User Registration</t>
+  </si>
+  <si>
+    <t>[TC006] Register with valid details</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:06.408Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:10.483Z</t>
+  </si>
+  <si>
+    <t>4.08s</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>[TC007] Register with existing email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:10.551Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:14.767Z</t>
+  </si>
+  <si>
+    <t>4.22s</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>[TC008] Register with invalid email</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:14.925Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:18.333Z</t>
+  </si>
+  <si>
+    <t>3.41s</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>[TC009] Register with weak password</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:18.501Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:21.705Z</t>
+  </si>
+  <si>
+    <t>3.20s</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>[TC010] Register with missing mandatory fields</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:21.951Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:56.577Z</t>
+  </si>
+  <si>
+    <t>34.63s</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Module 3: Fraud Alert Detection</t>
+  </si>
+  <si>
+    <t>[TC011] Upload suspicious SMS content</t>
+  </si>
+  <si>
     <t>FAILED</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:07.333Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:11.846Z</t>
-  </si>
-  <si>
-    <t>3.50s</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>[TC002] Login with invalid credentials</t>
-  </si>
-  <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:11.923Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:15.591Z</t>
-  </si>
-  <si>
-    <t>3.67s</t>
-  </si>
-  <si>
-    <t>TC003</t>
-  </si>
-  <si>
-    <t>[TC003] Login with empty email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:15.975Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:19.403Z</t>
-  </si>
-  <si>
-    <t>3.43s</t>
-  </si>
-  <si>
-    <t>TC004</t>
-  </si>
-  <si>
-    <t>[TC004] Login with empty password</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:19.519Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:22.221Z</t>
-  </si>
-  <si>
-    <t>2.70s</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>[TC005] Forgot password flow</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:22.322Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:26.318Z</t>
+    <t>2026-08-20T09:22:57.048Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:06.522Z</t>
+  </si>
+  <si>
+    <t>8.63s</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>[TC012] Upload phishing message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:06.647Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:13.045Z</t>
+  </si>
+  <si>
+    <t>5.61s</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>[TC013] Upload safe banking message</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:13.152Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:19.455Z</t>
+  </si>
+  <si>
+    <t>5.50s</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>[TC014] Analyze suspicious URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:19.699Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:26.419Z</t>
+  </si>
+  <si>
+    <t>6.72s</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>[TC015] Analyze known phishing URL</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:26.599Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:32.275Z</t>
+  </si>
+  <si>
+    <t>5.68s</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Module 4: Safe Call Analysis</t>
+  </si>
+  <si>
+    <t>[TC016] Analyze legitimate phone number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:32.681Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:39.746Z</t>
+  </si>
+  <si>
+    <t>7.07s</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>[TC017] Analyze spam caller number</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:39.928Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:46.631Z</t>
+  </si>
+  <si>
+    <t>6.70s</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>[TC018] Analyze unknown caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:46.800Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:52.413Z</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>[TC019] Block suspicious caller</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:52.567Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:58.070Z</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>[TC020] View call analysis history</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:58.158Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:02.772Z</t>
+  </si>
+  <si>
+    <t>4.61s</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Module 5: Banking Awareness</t>
+  </si>
+  <si>
+    <t>[TC021] Open fraud awareness page</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:02.871Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:06.872Z</t>
   </si>
   <si>
     <t>4.00s</t>
   </si>
   <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>Module 2: User Registration</t>
-  </si>
-  <si>
-    <t>[TC006] Register with valid details</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:26.902Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:31.239Z</t>
-  </si>
-  <si>
-    <t>3.46s</t>
-  </si>
-  <si>
-    <t>TC007</t>
-  </si>
-  <si>
-    <t>[TC007] Register with existing email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:31.342Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:34.962Z</t>
-  </si>
-  <si>
-    <t>3.62s</t>
-  </si>
-  <si>
-    <t>TC008</t>
-  </si>
-  <si>
-    <t>[TC008] Register with invalid email</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:35.134Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:39.206Z</t>
-  </si>
-  <si>
-    <t>4.07s</t>
-  </si>
-  <si>
-    <t>TC009</t>
-  </si>
-  <si>
-    <t>[TC009] Register with weak password</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:39.341Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:42.980Z</t>
-  </si>
-  <si>
-    <t>3.64s</t>
-  </si>
-  <si>
-    <t>TC010</t>
-  </si>
-  <si>
-    <t>[TC010] Register with missing mandatory fields</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:43.045Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:47.430Z</t>
-  </si>
-  <si>
-    <t>4.38s</t>
-  </si>
-  <si>
-    <t>TC011</t>
-  </si>
-  <si>
-    <t>Module 3: Fraud Alert Detection</t>
-  </si>
-  <si>
-    <t>[TC011] Upload suspicious SMS content</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:47.499Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:54.535Z</t>
-  </si>
-  <si>
-    <t>5.89s</t>
-  </si>
-  <si>
-    <t>TC012</t>
-  </si>
-  <si>
-    <t>[TC012] Upload phishing message</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:54.652Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:02.007Z</t>
-  </si>
-  <si>
-    <t>6.63s</t>
-  </si>
-  <si>
-    <t>TC013</t>
-  </si>
-  <si>
-    <t>[TC013] Upload safe banking message</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:02.408Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:11.223Z</t>
-  </si>
-  <si>
-    <t>7.74s</t>
-  </si>
-  <si>
-    <t>TC014</t>
-  </si>
-  <si>
-    <t>[TC014] Analyze suspicious URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:11.392Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:18.415Z</t>
-  </si>
-  <si>
-    <t>7.02s</t>
-  </si>
-  <si>
-    <t>TC015</t>
-  </si>
-  <si>
-    <t>[TC015] Analyze known phishing URL</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:18.875Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:24.490Z</t>
-  </si>
-  <si>
-    <t>5.61s</t>
-  </si>
-  <si>
-    <t>TC016</t>
-  </si>
-  <si>
-    <t>Module 4: Safe Call Analysis</t>
-  </si>
-  <si>
-    <t>[TC016] Analyze legitimate phone number</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:24.815Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:31.532Z</t>
-  </si>
-  <si>
-    <t>6.72s</t>
-  </si>
-  <si>
-    <t>TC017</t>
-  </si>
-  <si>
-    <t>[TC017] Analyze spam caller number</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:31.681Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:36.877Z</t>
-  </si>
-  <si>
-    <t>5.20s</t>
-  </si>
-  <si>
-    <t>TC018</t>
-  </si>
-  <si>
-    <t>[TC018] Analyze unknown caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:37.037Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:43.208Z</t>
-  </si>
-  <si>
-    <t>6.17s</t>
-  </si>
-  <si>
-    <t>TC019</t>
-  </si>
-  <si>
-    <t>[TC019] Block suspicious caller</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:43.367Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:47.830Z</t>
-  </si>
-  <si>
-    <t>4.46s</t>
-  </si>
-  <si>
-    <t>TC020</t>
-  </si>
-  <si>
-    <t>[TC020] View call analysis history</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:47.990Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:53.335Z</t>
-  </si>
-  <si>
-    <t>5.34s</t>
-  </si>
-  <si>
-    <t>TC021</t>
-  </si>
-  <si>
-    <t>Module 5: Banking Awareness</t>
-  </si>
-  <si>
-    <t>[TC021] Open fraud awareness page</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:53.476Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:57.405Z</t>
-  </si>
-  <si>
-    <t>3.93s</t>
-  </si>
-  <si>
     <t>TC022</t>
   </si>
   <si>
     <t>[TC022] Load educational content</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:57.497Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:02.821Z</t>
-  </si>
-  <si>
-    <t>5.32s</t>
+    <t>2026-08-20T09:24:06.993Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:11.581Z</t>
+  </si>
+  <si>
+    <t>4.59s</t>
   </si>
   <si>
     <t>TC023</t>
@@ -443,13 +437,13 @@
     <t>[TC023] Play awareness video</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:03.109Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:09.143Z</t>
-  </si>
-  <si>
-    <t>6.03s</t>
+    <t>2026-08-20T09:24:11.714Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:16.113Z</t>
+  </si>
+  <si>
+    <t>4.40s</t>
   </si>
   <si>
     <t>TC024</t>
@@ -458,13 +452,13 @@
     <t>[TC024] Search awareness topics</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:09.565Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:14.250Z</t>
-  </si>
-  <si>
-    <t>4.68s</t>
+    <t>2026-08-20T09:24:16.218Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:26.490Z</t>
+  </si>
+  <si>
+    <t>10.27s</t>
   </si>
   <si>
     <t>TC025</t>
@@ -473,13 +467,13 @@
     <t>[TC025] Bookmark awareness article</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:14.379Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:21.724Z</t>
-  </si>
-  <si>
-    <t>7.34s</t>
+    <t>2026-08-20T09:24:26.817Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:45.440Z</t>
+  </si>
+  <si>
+    <t>18.62s</t>
   </si>
   <si>
     <t>TC026</t>
@@ -491,13 +485,13 @@
     <t>[TC026] Dashboard loads successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:22.015Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:27.477Z</t>
-  </si>
-  <si>
-    <t>5.46s</t>
+    <t>2026-08-20T09:24:45.837Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:49.277Z</t>
+  </si>
+  <si>
+    <t>3.44s</t>
   </si>
   <si>
     <t>TC027</t>
@@ -506,13 +500,13 @@
     <t>[TC027] Threat statistics displayed</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:27.680Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:36.531Z</t>
-  </si>
-  <si>
-    <t>8.85s</t>
+    <t>2026-08-20T09:24:49.407Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:53.178Z</t>
+  </si>
+  <si>
+    <t>3.77s</t>
   </si>
   <si>
     <t>TC028</t>
@@ -521,13 +515,13 @@
     <t>[TC028] Filter analytics</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:37.146Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:46.624Z</t>
-  </si>
-  <si>
-    <t>9.48s</t>
+    <t>2026-08-20T09:24:53.258Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:01.131Z</t>
+  </si>
+  <si>
+    <t>7.87s</t>
   </si>
   <si>
     <t>TC029</t>
@@ -536,13 +530,13 @@
     <t>[TC029] Monthly fraud report loads</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:46.703Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:21:01.638Z</t>
-  </si>
-  <si>
-    <t>14.94s</t>
+    <t>2026-08-20T09:25:01.289Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:13.861Z</t>
+  </si>
+  <si>
+    <t>12.57s</t>
   </si>
   <si>
     <t>TC030</t>
@@ -551,13 +545,13 @@
     <t>[TC030] Export analytics report</t>
   </si>
   <si>
-    <t>2026-08-20T09:21:01.767Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:21:06.576Z</t>
-  </si>
-  <si>
-    <t>4.81s</t>
+    <t>2026-08-20T09:25:13.980Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:19.912Z</t>
+  </si>
+  <si>
+    <t>5.93s</t>
   </si>
   <si>
     <t>Failure Reason</t>
@@ -572,28 +566,16 @@
     <t>expected false to be true</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_1__Authentication__TC001__Login_with_valid_credentials_1787217490833.png</t>
-  </si>
-  <si>
-    <t>http://localhost:5173/dashboard</t>
-  </si>
-  <si>
-    <t>expected 'http://localhost:5173/register' to include '/dashboard'</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_2__User_Registration__TC006__Register_with_valid_details_1787217510366.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217533391.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC011__Upload_suspicious_SMS_content_1787217785676.png</t>
   </si>
   <si>
     <t>http://localhost:5173/sms-scanner</t>
   </si>
   <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217541279.png</t>
-  </si>
-  <si>
-    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217550148.png</t>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC012__Upload_phishing_message_1787217792259.png</t>
+  </si>
+  <si>
+    <t>screenshots\fail_SafeBank_AI_E2E_Test_Suite_Module_3__Fraud_Alert_Detection__TC013__Upload_safe_banking_message_1787217798654.png</t>
   </si>
   <si>
     <t>Timestamp</t>
@@ -611,7 +593,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:09.054Z</t>
+    <t>2026-08-20T09:21:22.920Z</t>
   </si>
   <si>
     <t>Navigated to Login page</t>
@@ -623,58 +605,64 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-20T09:18:10.603Z</t>
+    <t>2026-08-20T09:21:23.872Z</t>
   </si>
   <si>
     <t>Submitted valid credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:14.142Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:15.216Z</t>
+    <t>2026-08-20T09:21:23.969Z</t>
+  </si>
+  <si>
+    <t>Successfully verified redirect to Dashboard</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:26.271Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:26.935Z</t>
   </si>
   <si>
     <t>Submitted incorrect credentials</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:15.590Z</t>
+    <t>2026-08-20T09:21:27.515Z</t>
   </si>
   <si>
     <t>Verified login error message displays correctly</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:18.474Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:19.250Z</t>
+    <t>2026-08-20T09:21:31.615Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:21:52.819Z</t>
   </si>
   <si>
     <t>Submitted empty email with password</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:19.402Z</t>
-  </si>
-  <si>
     <t>Verified empty email validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:21.443Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:22.119Z</t>
+    <t>2026-08-20T09:22:00.329Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:01.263Z</t>
   </si>
   <si>
     <t>Submitted valid email with empty password</t>
   </si>
   <si>
+    <t>2026-08-20T09:22:01.356Z</t>
+  </si>
+  <si>
     <t>Verified empty password validation triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:25.231Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:25.948Z</t>
+    <t>2026-08-20T09:22:04.915Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:05.997Z</t>
   </si>
   <si>
     <t>Triggered forgot password with email</t>
@@ -683,169 +671,166 @@
     <t>Verified forgot password success banner</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:29.195Z</t>
+    <t>2026-08-20T09:22:08.981Z</t>
   </si>
   <si>
     <t>Navigated to Register page</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:30.351Z</t>
-  </si>
-  <si>
-    <t>Submitted registration for new_86396@safebank.ai</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:33.424Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:34.578Z</t>
+    <t>2026-08-20T09:22:10.306Z</t>
+  </si>
+  <si>
+    <t>Submitted registration for new_6380@safebank.ai</t>
+  </si>
+  <si>
+    <t>Redirected to Dashboard after secure signup</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:12.799Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:14.547Z</t>
   </si>
   <si>
     <t>Submitted registration with existing email</t>
   </si>
   <si>
+    <t>2026-08-20T09:22:14.766Z</t>
+  </si>
+  <si>
     <t>Verified duplicate email registration error</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:37.866Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:39.083Z</t>
+    <t>2026-08-20T09:22:16.820Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:18.225Z</t>
   </si>
   <si>
     <t>Submitted registration with malformed email</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:39.205Z</t>
-  </si>
-  <si>
     <t>Verified invalid email pattern validation</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:41.660Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:42.870Z</t>
+    <t>2026-08-20T09:22:20.420Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:21.568Z</t>
   </si>
   <si>
     <t>Submitted registration with password too short</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:42.979Z</t>
-  </si>
-  <si>
     <t>Verified weak password warning trigger</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:45.788Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:18:47.173Z</t>
+    <t>2026-08-20T09:22:47.990Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:22:56.282Z</t>
   </si>
   <si>
     <t>Submitted empty registration fields</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:47.429Z</t>
+    <t>2026-08-20T09:22:56.576Z</t>
   </si>
   <si>
     <t>Verified all mandatory fields validation displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:51.917Z</t>
+    <t>2026-08-20T09:23:04.340Z</t>
   </si>
   <si>
     <t>Navigated to SMS Scanner page</t>
   </si>
   <si>
-    <t>2026-08-20T09:18:53.330Z</t>
+    <t>2026-08-20T09:23:05.624Z</t>
   </si>
   <si>
     <t>Submitted suspicious KYC spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:00.207Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:01.190Z</t>
+    <t>2026-08-20T09:23:11.150Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:12.204Z</t>
   </si>
   <si>
     <t>Submitted lottery phishing spam SMS content</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:08.721Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:10.089Z</t>
+    <t>2026-08-20T09:23:17.390Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:18.606Z</t>
   </si>
   <si>
     <t>Submitted clean SMS message</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:16.785Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:17.615Z</t>
+    <t>2026-08-20T09:23:24.517Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:25.578Z</t>
   </si>
   <si>
     <t>Submitted suspicious URL for analysis</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:18.414Z</t>
+    <t>2026-08-20T09:23:26.418Z</t>
   </si>
   <si>
     <t>Verified URL threat analysis completes successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:22.466Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:23.591Z</t>
+    <t>2026-08-20T09:23:30.233Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:31.443Z</t>
   </si>
   <si>
     <t>Submitted known phishing link URL</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:24.489Z</t>
-  </si>
-  <si>
     <t>Verified malicious threat flag alert triggers</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:30.011Z</t>
+    <t>2026-08-20T09:23:38.180Z</t>
   </si>
   <si>
     <t>Navigated to Call Analyzer page</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:30.766Z</t>
+    <t>2026-08-20T09:23:38.988Z</t>
   </si>
   <si>
     <t>Submitted legitimate phone number for scan</t>
   </si>
   <si>
+    <t>2026-08-20T09:23:39.745Z</t>
+  </si>
+  <si>
     <t>Verified legitimate number marked Safe</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:35.203Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:36.031Z</t>
+    <t>2026-08-20T09:23:45.229Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:45.826Z</t>
   </si>
   <si>
     <t>Submitted spam preset phone number for scan</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:36.876Z</t>
-  </si>
-  <si>
     <t>Verified spam preset marked Suspicious</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:41.791Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:42.462Z</t>
+    <t>2026-08-20T09:23:50.742Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:51.573Z</t>
   </si>
   <si>
     <t>Submitted unknown phone number for scan</t>
@@ -854,154 +839,151 @@
     <t>Verified call risk assessment generated and shown</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:46.920Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:47.740Z</t>
+    <t>2026-08-20T09:23:57.205Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:23:58.007Z</t>
   </si>
   <si>
     <t>Blocked phone number manually</t>
   </si>
   <si>
+    <t>2026-08-20T09:23:58.069Z</t>
+  </si>
+  <si>
     <t>Verified number successfully appended to Blocked List table</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:51.769Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:19:52.486Z</t>
+    <t>2026-08-20T09:24:01.473Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:01.911Z</t>
   </si>
   <si>
     <t>Scanned caller number to log history entry</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:53.334Z</t>
-  </si>
-  <si>
     <t>Verified scanned calls displays in Screening Logs</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:57.357Z</t>
+    <t>2026-08-20T09:24:06.861Z</t>
   </si>
   <si>
     <t>Navigated to Awareness page</t>
   </si>
   <si>
-    <t>2026-08-20T09:19:57.404Z</t>
+    <t>2026-08-20T09:24:06.871Z</t>
   </si>
   <si>
     <t>Verified page loaded successfully</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:02.255Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:02.820Z</t>
+    <t>2026-08-20T09:24:11.028Z</t>
   </si>
   <si>
     <t>Verified educational articles catalog displays</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:08.165Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:08.963Z</t>
+    <t>2026-08-20T09:24:14.935Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:15.932Z</t>
   </si>
   <si>
     <t>Clicked Play Video button</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:09.142Z</t>
+    <t>2026-08-20T09:24:16.112Z</t>
   </si>
   <si>
     <t>Verified video player status changed to Playing</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:13.540Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:14.205Z</t>
+    <t>2026-08-20T09:24:25.882Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:26.459Z</t>
   </si>
   <si>
     <t>Typed search query "OTP"</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:14.249Z</t>
-  </si>
-  <si>
     <t>Verified articles list filtered based on search query</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:19.317Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:21.051Z</t>
+    <t>2026-08-20T09:24:44.161Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:45.361Z</t>
   </si>
   <si>
     <t>Clicked bookmark action button on index 0</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:21.723Z</t>
-  </si>
-  <si>
     <t>Verified article added to Bookmarked Resources section</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:27.423Z</t>
+    <t>2026-08-20T09:24:49.241Z</t>
   </si>
   <si>
     <t>Navigated to Dashboard page</t>
   </si>
   <si>
+    <t>2026-08-20T09:24:49.276Z</t>
+  </si>
+  <si>
     <t>Verified security dashboard cards loaded</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:36.021Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:36.530Z</t>
+    <t>2026-08-20T09:24:53.045Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:24:53.177Z</t>
   </si>
   <si>
     <t>Verified metrics visible on telemetry cards</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:46.383Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:46.572Z</t>
+    <t>2026-08-20T09:25:00.791Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:01.040Z</t>
   </si>
   <si>
     <t>Changed statistics filter option to Last 30 Days</t>
   </si>
   <si>
+    <t>2026-08-20T09:25:01.130Z</t>
+  </si>
+  <si>
     <t>Verified threat statistics numbers change dynamically</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:53.934Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:20:55.693Z</t>
+    <t>2026-08-20T09:25:05.342Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:07.552Z</t>
   </si>
   <si>
     <t>Opened monthly report modal</t>
   </si>
   <si>
-    <t>2026-08-20T09:20:55.908Z</t>
+    <t>2026-08-20T09:25:08.280Z</t>
   </si>
   <si>
     <t>Closed monthly report modal</t>
   </si>
   <si>
-    <t>2026-08-20T09:21:01.637Z</t>
+    <t>2026-08-20T09:25:13.860Z</t>
   </si>
   <si>
     <t>Verified monthly intelligence report toggle details</t>
   </si>
   <si>
-    <t>2026-08-20T09:21:05.716Z</t>
-  </si>
-  <si>
-    <t>2026-08-20T09:21:06.382Z</t>
+    <t>2026-08-20T09:25:18.611Z</t>
+  </si>
+  <si>
+    <t>2026-08-20T09:25:19.535Z</t>
   </si>
   <si>
     <t>Clicked Export Report button</t>
@@ -1019,7 +1001,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>168.10s</t>
+    <t>233.46s</t>
   </si>
 </sst>
 </file>
@@ -1524,7 +1506,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1532,7 +1514,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1617,7 +1599,7 @@
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1644,241 +1626,241 @@
         <v>25</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>80</v>
@@ -1895,7 +1877,7 @@
         <v>83</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>84</v>
@@ -1904,7 +1886,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>85</v>
@@ -1921,7 +1903,7 @@
         <v>88</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>89</v>
@@ -1930,7 +1912,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>90</v>
@@ -1947,7 +1929,7 @@
         <v>93</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>94</v>
@@ -1956,7 +1938,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>95</v>
@@ -1973,7 +1955,7 @@
         <v>98</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>99</v>
@@ -1982,7 +1964,7 @@
         <v>25</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>100</v>
@@ -2008,7 +1990,7 @@
         <v>25</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>106</v>
@@ -2034,7 +2016,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>111</v>
@@ -2060,7 +2042,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>116</v>
@@ -2069,319 +2051,319 @@
         <v>117</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>118</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="H20" s="2" t="s">
-        <v>123</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>104</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F24" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F25" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F30" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F31" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2392,7 +2374,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2406,101 +2388,67 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="7" t="s">
         <v>184</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2511,7 +2459,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2523,1413 +2471,1447 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>199</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>214</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>44</v>
+        <v>210</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>220</v>
+        <v>193</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>215</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>222</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>227</v>
+        <v>54</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>60</v>
+        <v>223</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>236</v>
+        <v>64</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>241</v>
+        <v>69</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>244</v>
+        <v>219</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>267</v>
+        <v>101</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>107</v>
+        <v>260</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>274</v>
+        <v>261</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>276</v>
+        <v>112</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>117</v>
+        <v>270</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="52" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>280</v>
+        <v>117</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>122</v>
+        <v>274</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>282</v>
+        <v>261</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="55" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>287</v>
+        <v>261</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="58" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>290</v>
+        <v>125</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="59" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="60" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="61" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>296</v>
+        <v>136</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="63" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="64" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="65" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="66" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="67" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="69" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="71" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="72" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="73" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="74" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="75" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="76" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>169</v>
+        <v>309</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>319</v>
+        <v>303</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="77" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>311</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="78" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="79" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>324</v>
+        <v>303</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="80" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>32</v>
+        <v>194</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>200</v>
+        <v>26</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="83" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>179</v>
+        <v>321</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C83" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="D83" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>201</v>
+      <c r="B85" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3952,7 +3934,7 @@
         <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3961,10 +3943,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3975,16 +3957,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>